<commit_message>
fixed the template format
</commit_message>
<xml_diff>
--- a/public/templates/CArm_Template.xlsx
+++ b/public/templates/CArm_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROJECTS\anteso\anteso-frontend\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA05D2C5-F0E8-4AC8-94E3-23A40E3B52D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F76839B4-2B8A-403A-82A5-8E48BA88881C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Data" sheetId="1" r:id="rId1"/>
@@ -21,459 +21,231 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="224">
-  <si>
-    <t>Field Name</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Description / Instructions</t>
-  </si>
-  <si>
-    <t>========== ACCURACY OF IRRADIATION TIME ==========</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="145">
+  <si>
+    <t>TEST: ACCURACY OF IRRADIATION TIME</t>
+  </si>
+  <si>
+    <t>FCD</t>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
+  <si>
+    <t>kV</t>
+  </si>
+  <si>
+    <t>80</t>
+  </si>
+  <si>
+    <t>mA</t>
+  </si>
+  <si>
+    <t>Set Time (ms)</t>
+  </si>
+  <si>
+    <t>Measured Time (ms)</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>Section separator – do not edit</t>
-  </si>
-  <si>
-    <t>TestConditions_FCD</t>
-  </si>
-  <si>
-    <t>100</t>
-  </si>
-  <si>
-    <t>Focus-to-detector distance (cm)</t>
-  </si>
-  <si>
-    <t>TestConditions_kV</t>
-  </si>
-  <si>
-    <t>80</t>
-  </si>
-  <si>
-    <t>kV</t>
-  </si>
-  <si>
-    <t>TestConditions_ma</t>
-  </si>
-  <si>
-    <t>mA</t>
-  </si>
-  <si>
-    <t>IrradiationTime_SetTime</t>
-  </si>
-  <si>
-    <t>Set time (ms)</t>
-  </si>
-  <si>
-    <t>IrradiationTime_MeasuredTime</t>
-  </si>
-  <si>
-    <t>Measured time (ms)</t>
-  </si>
-  <si>
     <t>200</t>
   </si>
   <si>
     <t>400</t>
   </si>
   <si>
-    <t>Tolerance_Operator</t>
+    <t>Tolerance</t>
   </si>
   <si>
     <t>&lt;=</t>
   </si>
   <si>
-    <t>Operator: &lt;=, &gt;=, =</t>
-  </si>
-  <si>
-    <t>Tolerance_Value</t>
+    <t>10%</t>
+  </si>
+  <si>
+    <t>TEST: TOTAL FILTRATION AND ACCURACY OF OPERATING POTENTIAL</t>
+  </si>
+  <si>
+    <t>Applied kVp</t>
+  </si>
+  <si>
+    <t>Meas 1 (50 mA)</t>
+  </si>
+  <si>
+    <t>Meas 2 (100 mA)</t>
+  </si>
+  <si>
+    <t>Average kVp</t>
+  </si>
+  <si>
+    <t>Remarks</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>Total Filtration</t>
+  </si>
+  <si>
+    <t>Measured (mm Al)</t>
+  </si>
+  <si>
+    <t>Required (mm Al)</t>
+  </si>
+  <si>
+    <t>At kVp</t>
+  </si>
+  <si>
+    <t>TotalFiltration</t>
+  </si>
+  <si>
+    <t>2.5</t>
+  </si>
+  <si>
+    <t>TEST: CONSISTENCY OF RADIATION OUTPUT</t>
+  </si>
+  <si>
+    <t>FFD (cm)</t>
+  </si>
+  <si>
+    <t>Time (ms)</t>
+  </si>
+  <si>
+    <t>Meas 1</t>
+  </si>
+  <si>
+    <t>Meas 2</t>
+  </si>
+  <si>
+    <t>Meas 3</t>
+  </si>
+  <si>
+    <t>Mean</t>
+  </si>
+  <si>
+    <t>CoV</t>
+  </si>
+  <si>
+    <t>Tolerance (CoV)</t>
+  </si>
+  <si>
+    <t>0.02</t>
+  </si>
+  <si>
+    <t>TEST: LOW CONTRAST RESOLUTION</t>
+  </si>
+  <si>
+    <t>Smallest Hole Size (mm)</t>
+  </si>
+  <si>
+    <t>Recommended Standard</t>
+  </si>
+  <si>
+    <t>TEST: HIGH CONTRAST RESOLUTION</t>
+  </si>
+  <si>
+    <t>Line Pairs per mm (Lp/mm)</t>
+  </si>
+  <si>
+    <t>TEST: EXPOSURE RATE AT TABLE TOP</t>
+  </si>
+  <si>
+    <t>AEC Tolerance (%)</t>
+  </si>
+  <si>
+    <t>Non-AEC Tolerance (%)</t>
+  </si>
+  <si>
+    <t>Min Focus Distance (cm)</t>
+  </si>
+  <si>
+    <t>Distance (cm)</t>
+  </si>
+  <si>
+    <t>mR 1</t>
+  </si>
+  <si>
+    <t>mR 2</t>
+  </si>
+  <si>
+    <t>mR 3</t>
+  </si>
+  <si>
+    <t>TEST: TUBE HOUSING LEAKAGE</t>
+  </si>
+  <si>
+    <t>FCD (cm)</t>
+  </si>
+  <si>
+    <t>Time (min)</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Workload</t>
+  </si>
+  <si>
+    <t>1000</t>
+  </si>
+  <si>
+    <t>Tolerance (mGy/h)</t>
+  </si>
+  <si>
+    <t>1.0</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>Left</t>
+  </si>
+  <si>
+    <t>Right</t>
+  </si>
+  <si>
+    <t>Front</t>
+  </si>
+  <si>
+    <t>Back</t>
+  </si>
+  <si>
+    <t>Top</t>
+  </si>
+  <si>
+    <t>Tube</t>
+  </si>
+  <si>
+    <t>Collimator</t>
+  </si>
+  <si>
+    <t>TEST: LINEARITY OF mA LOADING</t>
+  </si>
+  <si>
+    <t>mA Station</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>Tolerance (CoL)</t>
+  </si>
+  <si>
+    <t>0.1</t>
+  </si>
+  <si>
+    <t>TEST: LINEARITY OF mAs LOADING</t>
+  </si>
+  <si>
+    <t>mAs</t>
+  </si>
+  <si>
+    <t>5</t>
   </si>
   <si>
     <t>10</t>
-  </si>
-  <si>
-    <t>Tolerance value (%)</t>
-  </si>
-  <si>
-    <t>========== TOTAL FILTRATION ==========</t>
-  </si>
-  <si>
-    <t>mAStations</t>
-  </si>
-  <si>
-    <t>50 mA</t>
-  </si>
-  <si>
-    <t>mA station header</t>
-  </si>
-  <si>
-    <t>100 mA</t>
-  </si>
-  <si>
-    <t>Tolerance_Sign</t>
-  </si>
-  <si>
-    <t>±</t>
-  </si>
-  <si>
-    <t>±, + or -</t>
-  </si>
-  <si>
-    <t>2.0</t>
-  </si>
-  <si>
-    <t>Tolerance in kV</t>
-  </si>
-  <si>
-    <t>TotalFiltration_Measured</t>
-  </si>
-  <si>
-    <t>Measured total filtration (mm Al)</t>
-  </si>
-  <si>
-    <t>TotalFiltration_Required</t>
-  </si>
-  <si>
-    <t>2.5</t>
-  </si>
-  <si>
-    <t>Required minimum (mm Al)</t>
-  </si>
-  <si>
-    <t>Measurement_AppliedKvp</t>
-  </si>
-  <si>
-    <t>60</t>
-  </si>
-  <si>
-    <t>Applied kVp</t>
-  </si>
-  <si>
-    <t>Measurement_Meas1</t>
-  </si>
-  <si>
-    <t>Measured at station 1</t>
-  </si>
-  <si>
-    <t>Measurement_Meas2</t>
-  </si>
-  <si>
-    <t>Measured at station 2</t>
-  </si>
-  <si>
-    <t>Measurement_AverageKvp</t>
-  </si>
-  <si>
-    <t>Average kVp</t>
-  </si>
-  <si>
-    <t>========== CONSISTENCY OF RADIATION OUTPUT ==========</t>
-  </si>
-  <si>
-    <t>Parameters_FFD</t>
-  </si>
-  <si>
-    <t>FFD (cm)</t>
-  </si>
-  <si>
-    <t>Parameters_Time</t>
-  </si>
-  <si>
-    <t>Time (ms)</t>
-  </si>
-  <si>
-    <t>Output_Tolerance</t>
-  </si>
-  <si>
-    <t>0.02</t>
-  </si>
-  <si>
-    <t>CoV tolerance</t>
-  </si>
-  <si>
-    <t>Header_1</t>
-  </si>
-  <si>
-    <t>Meas 1</t>
-  </si>
-  <si>
-    <t>Measurement column header</t>
-  </si>
-  <si>
-    <t>Header_2</t>
-  </si>
-  <si>
-    <t>Meas 2</t>
-  </si>
-  <si>
-    <t>Header_3</t>
-  </si>
-  <si>
-    <t>Meas 3</t>
-  </si>
-  <si>
-    <t>Output_kV</t>
-  </si>
-  <si>
-    <t>Output_mA</t>
-  </si>
-  <si>
-    <t>Output_Meas1</t>
-  </si>
-  <si>
-    <t>Measurement 1</t>
-  </si>
-  <si>
-    <t>Output_Meas2</t>
-  </si>
-  <si>
-    <t>Measurement 2</t>
-  </si>
-  <si>
-    <t>Output_Meas3</t>
-  </si>
-  <si>
-    <t>Measurement 3</t>
-  </si>
-  <si>
-    <t>========== LOW CONTRAST RESOLUTION ==========</t>
-  </si>
-  <si>
-    <t>LowContrast_HoleSize</t>
-  </si>
-  <si>
-    <t>Smallest hole size (mm)</t>
-  </si>
-  <si>
-    <t>LowContrast_Standard</t>
-  </si>
-  <si>
-    <t>Recommended standard</t>
-  </si>
-  <si>
-    <t>========== HIGH CONTRAST RESOLUTION ==========</t>
-  </si>
-  <si>
-    <t>HighContrast_LpMm</t>
-  </si>
-  <si>
-    <t>Line pairs per mm</t>
-  </si>
-  <si>
-    <t>========== EXPOSURE RATE AT TABLE TOP ==========</t>
-  </si>
-  <si>
-    <t>ExposureRate_AecTolerance</t>
-  </si>
-  <si>
-    <t>AEC tolerance</t>
-  </si>
-  <si>
-    <t>ExposureRate_NonAecTolerance</t>
-  </si>
-  <si>
-    <t>Non-AEC tolerance</t>
-  </si>
-  <si>
-    <t>ExposureRate_MinFocusDistance</t>
-  </si>
-  <si>
-    <t>Min focus distance (cm)</t>
-  </si>
-  <si>
-    <t>ExposureRate_Distance</t>
-  </si>
-  <si>
-    <t>Distance (cm)</t>
-  </si>
-  <si>
-    <t>ExposureRate_Meas1</t>
-  </si>
-  <si>
-    <t>ExposureRate_Meas2</t>
-  </si>
-  <si>
-    <t>ExposureRate_Meas3</t>
-  </si>
-  <si>
-    <t>========== TUBE HOUSING LEAKAGE ==========</t>
-  </si>
-  <si>
-    <t>Leakage_FCD</t>
-  </si>
-  <si>
-    <t>FCD (cm)</t>
-  </si>
-  <si>
-    <t>Leakage_kV</t>
-  </si>
-  <si>
-    <t>Leakage_mA</t>
-  </si>
-  <si>
-    <t>Leakage_Time</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>Time (min)</t>
-  </si>
-  <si>
-    <t>Leakage_Workload</t>
-  </si>
-  <si>
-    <t>1000</t>
-  </si>
-  <si>
-    <t>Workload</t>
-  </si>
-  <si>
-    <t>Leakage_ToleranceValue</t>
-  </si>
-  <si>
-    <t>1.0</t>
-  </si>
-  <si>
-    <t>Tolerance value</t>
-  </si>
-  <si>
-    <t>Leakage_ToleranceOperator</t>
-  </si>
-  <si>
-    <t>less than or equal to</t>
-  </si>
-  <si>
-    <t>Tolerance operator</t>
-  </si>
-  <si>
-    <t>Leakage_Tube_Left</t>
-  </si>
-  <si>
-    <t>Tube – Left (mR/h)</t>
-  </si>
-  <si>
-    <t>Leakage_Tube_Right</t>
-  </si>
-  <si>
-    <t>Tube – Right</t>
-  </si>
-  <si>
-    <t>Leakage_Tube_Front</t>
-  </si>
-  <si>
-    <t>Tube – Front</t>
-  </si>
-  <si>
-    <t>Leakage_Tube_Back</t>
-  </si>
-  <si>
-    <t>Tube – Back</t>
-  </si>
-  <si>
-    <t>Leakage_Tube_Top</t>
-  </si>
-  <si>
-    <t>Tube – Top</t>
-  </si>
-  <si>
-    <t>Leakage_Collimator_Left</t>
-  </si>
-  <si>
-    <t>Collimator – Left</t>
-  </si>
-  <si>
-    <t>Leakage_Collimator_Right</t>
-  </si>
-  <si>
-    <t>Collimator – Right</t>
-  </si>
-  <si>
-    <t>Leakage_Collimator_Front</t>
-  </si>
-  <si>
-    <t>Collimator – Front</t>
-  </si>
-  <si>
-    <t>Leakage_Collimator_Back</t>
-  </si>
-  <si>
-    <t>Collimator – Back</t>
-  </si>
-  <si>
-    <t>Leakage_Collimator_Top</t>
-  </si>
-  <si>
-    <t>Collimator – Top</t>
-  </si>
-  <si>
-    <t>========== LINEARITY OF MA LOADING ==========</t>
-  </si>
-  <si>
-    <t>Linearity_FCD</t>
-  </si>
-  <si>
-    <t>Linearity_kV</t>
-  </si>
-  <si>
-    <t>Linearity_Time</t>
-  </si>
-  <si>
-    <t>Linearity_Tolerance</t>
-  </si>
-  <si>
-    <t>0.1</t>
-  </si>
-  <si>
-    <t>Tolerance</t>
-  </si>
-  <si>
-    <t>Measurement header</t>
-  </si>
-  <si>
-    <t>Linearity_mA</t>
-  </si>
-  <si>
-    <t>50</t>
-  </si>
-  <si>
-    <t>mA station</t>
-  </si>
-  <si>
-    <t>Linearity_Meas1</t>
-  </si>
-  <si>
-    <t>Measured 1</t>
-  </si>
-  <si>
-    <t>Linearity_Meas2</t>
-  </si>
-  <si>
-    <t>Measured 2</t>
-  </si>
-  <si>
-    <t>Linearity_Meas3</t>
-  </si>
-  <si>
-    <t>Measured 3</t>
-  </si>
-  <si>
-    <t>========== LINEARITY OF MAS LOADING ==========</t>
-  </si>
-  <si>
-    <t>Linearity_mAs</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>mAs value</t>
   </si>
   <si>
     <t>Name of the Hospital</t>
@@ -668,9 +440,6 @@
     <t>mAmin in 1 hr</t>
   </si>
   <si>
-    <t>Location</t>
-  </si>
-  <si>
     <t>mR/h</t>
   </si>
   <si>
@@ -693,12 +462,6 @@
   </si>
   <si>
     <t>TOP</t>
-  </si>
-  <si>
-    <t>Tube</t>
-  </si>
-  <si>
-    <t>Collimator</t>
   </si>
   <si>
     <t>Tolerance: Tube Leakage &lt; 1 mGy in one hour</t>
@@ -727,8 +490,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="165" formatCode="0.000"/>
-    <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -1800,13 +1563,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1815,13 +1578,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1833,13 +1596,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="7" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1923,7 +1686,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1935,13 +1698,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="8" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1953,10 +1716,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="8" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2085,7 +1848,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2552,1245 +2315,634 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C111"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:J56"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="54.296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.3984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.19921875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="58.69921875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.19921875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.3984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.69921875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.8984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="1.8984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.09765625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.8984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="B2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="C2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="F2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>9</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>10</v>
       </c>
-      <c r="C4" t="s">
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="B7" t="s">
         <v>12</v>
       </c>
-      <c r="B5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="C7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>14</v>
       </c>
-      <c r="B6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" t="s">
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="B10" t="s">
         <v>16</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" t="s">
+        <v>18</v>
+      </c>
+      <c r="E10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>4</v>
       </c>
-      <c r="C7" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="B12" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B13" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" t="s">
+        <v>26</v>
+      </c>
+      <c r="D15" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" t="s">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B18" t="s">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>29</v>
+      </c>
+      <c r="D18" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>3</v>
+      </c>
+      <c r="B19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" t="s">
+        <v>30</v>
+      </c>
+      <c r="D19" t="s">
+        <v>31</v>
+      </c>
+      <c r="E19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G19" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
         <v>4</v>
       </c>
-      <c r="C9" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" t="s">
-        <v>4</v>
-      </c>
-      <c r="C11" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" t="s">
-        <v>21</v>
-      </c>
-      <c r="C12" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>23</v>
-      </c>
-      <c r="B13" t="s">
-        <v>24</v>
-      </c>
-      <c r="C13" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" t="s">
-        <v>4</v>
-      </c>
-      <c r="C14" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>27</v>
-      </c>
-      <c r="B15" t="s">
-        <v>28</v>
-      </c>
-      <c r="C15" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>27</v>
-      </c>
-      <c r="B16" t="s">
-        <v>30</v>
-      </c>
-      <c r="C16" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>31</v>
-      </c>
-      <c r="B17" t="s">
-        <v>32</v>
-      </c>
-      <c r="C17" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>23</v>
-      </c>
-      <c r="B18" t="s">
-        <v>34</v>
-      </c>
-      <c r="C18" t="s">
+      <c r="B20" t="s">
+        <v>2</v>
+      </c>
+      <c r="C20" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" t="s">
+        <v>8</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>8</v>
+      </c>
+      <c r="G20" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>2</v>
+      </c>
+      <c r="B21" t="s">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" t="s">
+        <v>8</v>
+      </c>
+      <c r="E21" t="s">
+        <v>8</v>
+      </c>
+      <c r="F21" t="s">
+        <v>8</v>
+      </c>
+      <c r="G21" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
+      <c r="B22" t="s">
         <v>36</v>
       </c>
-      <c r="B19" t="s">
-        <v>4</v>
-      </c>
-      <c r="C19" t="s">
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
         <v>38</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B25" t="s">
         <v>39</v>
       </c>
-      <c r="C20" t="s">
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>8</v>
+      </c>
+      <c r="B26" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>41</v>
-      </c>
-      <c r="B21" t="s">
-        <v>42</v>
-      </c>
-      <c r="C21" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>44</v>
-      </c>
-      <c r="B22" t="s">
-        <v>4</v>
-      </c>
-      <c r="C22" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>46</v>
-      </c>
-      <c r="B23" t="s">
-        <v>4</v>
-      </c>
-      <c r="C23" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>48</v>
-      </c>
-      <c r="B24" t="s">
-        <v>4</v>
-      </c>
-      <c r="C24" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>41</v>
-      </c>
-      <c r="B25" t="s">
-        <v>10</v>
-      </c>
-      <c r="C25" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>44</v>
-      </c>
-      <c r="B26" t="s">
-        <v>4</v>
-      </c>
-      <c r="C26" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>46</v>
-      </c>
-      <c r="B27" t="s">
-        <v>4</v>
-      </c>
-      <c r="C27" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>48</v>
-      </c>
-      <c r="B28" t="s">
-        <v>4</v>
-      </c>
-      <c r="C28" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>41</v>
       </c>
-      <c r="B29" t="s">
-        <v>7</v>
-      </c>
-      <c r="C29" t="s">
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>43</v>
+      </c>
+      <c r="B33" t="s">
+        <v>8</v>
+      </c>
+      <c r="C33" t="s">
+        <v>44</v>
+      </c>
+      <c r="D33" t="s">
+        <v>8</v>
+      </c>
+      <c r="E33" t="s">
+        <v>45</v>
+      </c>
+      <c r="F33" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>46</v>
+      </c>
+      <c r="B34" t="s">
+        <v>47</v>
+      </c>
+      <c r="C34" t="s">
+        <v>48</v>
+      </c>
+      <c r="D34" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>2</v>
+      </c>
+      <c r="B35" t="s">
+        <v>8</v>
+      </c>
+      <c r="C35" t="s">
+        <v>8</v>
+      </c>
+      <c r="D35" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>51</v>
+      </c>
+      <c r="B38" t="s">
+        <v>2</v>
+      </c>
+      <c r="C38" t="s">
+        <v>3</v>
+      </c>
+      <c r="D38" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>44</v>
-      </c>
-      <c r="B30" t="s">
+      <c r="E38" t="s">
+        <v>5</v>
+      </c>
+      <c r="F38" t="s">
+        <v>2</v>
+      </c>
+      <c r="G38" t="s">
+        <v>52</v>
+      </c>
+      <c r="H38" t="s">
+        <v>53</v>
+      </c>
+      <c r="I38" t="s">
+        <v>54</v>
+      </c>
+      <c r="J38" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>56</v>
+      </c>
+      <c r="B39" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>58</v>
+      </c>
+      <c r="B40" t="s">
+        <v>59</v>
+      </c>
+      <c r="C40" t="s">
+        <v>60</v>
+      </c>
+      <c r="D40" t="s">
+        <v>61</v>
+      </c>
+      <c r="E40" t="s">
+        <v>62</v>
+      </c>
+      <c r="F40" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>64</v>
+      </c>
+      <c r="B41" t="s">
+        <v>8</v>
+      </c>
+      <c r="C41" t="s">
+        <v>8</v>
+      </c>
+      <c r="D41" t="s">
+        <v>8</v>
+      </c>
+      <c r="E41" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42" t="s">
+        <v>8</v>
+      </c>
+      <c r="C42" t="s">
+        <v>8</v>
+      </c>
+      <c r="D42" t="s">
+        <v>8</v>
+      </c>
+      <c r="E42" t="s">
+        <v>8</v>
+      </c>
+      <c r="F42" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>51</v>
+      </c>
+      <c r="B45" t="s">
+        <v>2</v>
+      </c>
+      <c r="C45" t="s">
+        <v>3</v>
+      </c>
+      <c r="D45" t="s">
         <v>4</v>
       </c>
-      <c r="C30" t="s">
+      <c r="E45" t="s">
+        <v>29</v>
+      </c>
+      <c r="F45" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>67</v>
+      </c>
+      <c r="B46" t="s">
+        <v>30</v>
+      </c>
+      <c r="C46" t="s">
+        <v>31</v>
+      </c>
+      <c r="D46" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>68</v>
+      </c>
+      <c r="B47" t="s">
+        <v>8</v>
+      </c>
+      <c r="C47" t="s">
+        <v>8</v>
+      </c>
+      <c r="D47" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>2</v>
+      </c>
+      <c r="B48" t="s">
+        <v>8</v>
+      </c>
+      <c r="C48" t="s">
+        <v>8</v>
+      </c>
+      <c r="D48" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>69</v>
+      </c>
+      <c r="B49" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>51</v>
+      </c>
+      <c r="B52" t="s">
+        <v>2</v>
+      </c>
+      <c r="C52" t="s">
+        <v>3</v>
+      </c>
+      <c r="D52" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>46</v>
-      </c>
-      <c r="B31" t="s">
-        <v>4</v>
-      </c>
-      <c r="C31" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>48</v>
-      </c>
-      <c r="B32" t="s">
-        <v>4</v>
-      </c>
-      <c r="C32" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>50</v>
-      </c>
-      <c r="B33" t="s">
-        <v>4</v>
-      </c>
-      <c r="C33" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>51</v>
-      </c>
-      <c r="B34" t="s">
-        <v>7</v>
-      </c>
-      <c r="C34" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>53</v>
-      </c>
-      <c r="B35" t="s">
-        <v>7</v>
-      </c>
-      <c r="C35" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>55</v>
-      </c>
-      <c r="B36" t="s">
-        <v>56</v>
-      </c>
-      <c r="C36" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
-        <v>58</v>
-      </c>
-      <c r="B37" t="s">
-        <v>59</v>
-      </c>
-      <c r="C37" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
-        <v>61</v>
-      </c>
-      <c r="B38" t="s">
-        <v>62</v>
-      </c>
-      <c r="C38" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
-        <v>63</v>
-      </c>
-      <c r="B39" t="s">
-        <v>64</v>
-      </c>
-      <c r="C39" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
-        <v>65</v>
-      </c>
-      <c r="B40" t="s">
-        <v>10</v>
-      </c>
-      <c r="C40" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
-        <v>66</v>
-      </c>
-      <c r="B41" t="s">
-        <v>7</v>
-      </c>
-      <c r="C41" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A42" t="s">
-        <v>67</v>
-      </c>
-      <c r="B42" t="s">
-        <v>4</v>
-      </c>
-      <c r="C42" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>72</v>
+      </c>
+      <c r="B53" t="s">
+        <v>30</v>
+      </c>
+      <c r="C53" t="s">
+        <v>31</v>
+      </c>
+      <c r="D53" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>73</v>
+      </c>
+      <c r="B54" t="s">
+        <v>8</v>
+      </c>
+      <c r="C54" t="s">
+        <v>8</v>
+      </c>
+      <c r="D54" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>74</v>
+      </c>
+      <c r="B55" t="s">
+        <v>8</v>
+      </c>
+      <c r="C55" t="s">
+        <v>8</v>
+      </c>
+      <c r="D55" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
         <v>69</v>
       </c>
-      <c r="B43" t="s">
-        <v>4</v>
-      </c>
-      <c r="C43" t="s">
+      <c r="B56" t="s">
         <v>70</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
-        <v>71</v>
-      </c>
-      <c r="B44" t="s">
-        <v>4</v>
-      </c>
-      <c r="C44" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
-        <v>65</v>
-      </c>
-      <c r="B45" t="s">
-        <v>7</v>
-      </c>
-      <c r="C45" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A46" t="s">
-        <v>66</v>
-      </c>
-      <c r="B46" t="s">
-        <v>7</v>
-      </c>
-      <c r="C46" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A47" t="s">
-        <v>67</v>
-      </c>
-      <c r="B47" t="s">
-        <v>4</v>
-      </c>
-      <c r="C47" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A48" t="s">
-        <v>69</v>
-      </c>
-      <c r="B48" t="s">
-        <v>4</v>
-      </c>
-      <c r="C48" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A49" t="s">
-        <v>71</v>
-      </c>
-      <c r="B49" t="s">
-        <v>4</v>
-      </c>
-      <c r="C49" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
-        <v>73</v>
-      </c>
-      <c r="B50" t="s">
-        <v>4</v>
-      </c>
-      <c r="C50" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A51" t="s">
-        <v>74</v>
-      </c>
-      <c r="B51" t="s">
-        <v>4</v>
-      </c>
-      <c r="C51" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A52" t="s">
-        <v>76</v>
-      </c>
-      <c r="B52" t="s">
-        <v>4</v>
-      </c>
-      <c r="C52" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A53" t="s">
-        <v>78</v>
-      </c>
-      <c r="B53" t="s">
-        <v>4</v>
-      </c>
-      <c r="C53" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A54" t="s">
-        <v>79</v>
-      </c>
-      <c r="B54" t="s">
-        <v>4</v>
-      </c>
-      <c r="C54" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A55" t="s">
-        <v>81</v>
-      </c>
-      <c r="B55" t="s">
-        <v>4</v>
-      </c>
-      <c r="C55" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A56" t="s">
-        <v>82</v>
-      </c>
-      <c r="B56" t="s">
-        <v>4</v>
-      </c>
-      <c r="C56" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A57" t="s">
-        <v>84</v>
-      </c>
-      <c r="B57" t="s">
-        <v>4</v>
-      </c>
-      <c r="C57" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A58" t="s">
-        <v>86</v>
-      </c>
-      <c r="B58" t="s">
-        <v>7</v>
-      </c>
-      <c r="C58" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A59" t="s">
-        <v>88</v>
-      </c>
-      <c r="B59" t="s">
-        <v>7</v>
-      </c>
-      <c r="C59" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A60" t="s">
-        <v>90</v>
-      </c>
-      <c r="B60" t="s">
-        <v>4</v>
-      </c>
-      <c r="C60" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A61" t="s">
-        <v>91</v>
-      </c>
-      <c r="B61" t="s">
-        <v>4</v>
-      </c>
-      <c r="C61" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A62" t="s">
-        <v>92</v>
-      </c>
-      <c r="B62" t="s">
-        <v>4</v>
-      </c>
-      <c r="C62" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A63" t="s">
-        <v>93</v>
-      </c>
-      <c r="B63" t="s">
-        <v>4</v>
-      </c>
-      <c r="C63" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A64" t="s">
-        <v>94</v>
-      </c>
-      <c r="B64" t="s">
-        <v>7</v>
-      </c>
-      <c r="C64" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A65" t="s">
-        <v>96</v>
-      </c>
-      <c r="B65" t="s">
-        <v>10</v>
-      </c>
-      <c r="C65" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A66" t="s">
-        <v>97</v>
-      </c>
-      <c r="B66" t="s">
-        <v>7</v>
-      </c>
-      <c r="C66" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A67" t="s">
-        <v>98</v>
-      </c>
-      <c r="B67" t="s">
-        <v>99</v>
-      </c>
-      <c r="C67" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A68" t="s">
-        <v>101</v>
-      </c>
-      <c r="B68" t="s">
-        <v>102</v>
-      </c>
-      <c r="C68" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A69" t="s">
-        <v>104</v>
-      </c>
-      <c r="B69" t="s">
-        <v>105</v>
-      </c>
-      <c r="C69" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A70" t="s">
-        <v>107</v>
-      </c>
-      <c r="B70" t="s">
-        <v>108</v>
-      </c>
-      <c r="C70" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A71" t="s">
-        <v>110</v>
-      </c>
-      <c r="B71" t="s">
-        <v>4</v>
-      </c>
-      <c r="C71" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A72" t="s">
-        <v>112</v>
-      </c>
-      <c r="B72" t="s">
-        <v>4</v>
-      </c>
-      <c r="C72" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A73" t="s">
-        <v>114</v>
-      </c>
-      <c r="B73" t="s">
-        <v>4</v>
-      </c>
-      <c r="C73" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A74" t="s">
-        <v>116</v>
-      </c>
-      <c r="B74" t="s">
-        <v>4</v>
-      </c>
-      <c r="C74" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A75" t="s">
-        <v>118</v>
-      </c>
-      <c r="B75" t="s">
-        <v>4</v>
-      </c>
-      <c r="C75" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A76" t="s">
-        <v>120</v>
-      </c>
-      <c r="B76" t="s">
-        <v>4</v>
-      </c>
-      <c r="C76" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A77" t="s">
-        <v>122</v>
-      </c>
-      <c r="B77" t="s">
-        <v>4</v>
-      </c>
-      <c r="C77" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A78" t="s">
-        <v>124</v>
-      </c>
-      <c r="B78" t="s">
-        <v>4</v>
-      </c>
-      <c r="C78" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A79" t="s">
-        <v>126</v>
-      </c>
-      <c r="B79" t="s">
-        <v>4</v>
-      </c>
-      <c r="C79" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A80" t="s">
-        <v>128</v>
-      </c>
-      <c r="B80" t="s">
-        <v>4</v>
-      </c>
-      <c r="C80" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A81" t="s">
-        <v>130</v>
-      </c>
-      <c r="B81" t="s">
-        <v>4</v>
-      </c>
-      <c r="C81" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A82" t="s">
-        <v>131</v>
-      </c>
-      <c r="B82" t="s">
-        <v>7</v>
-      </c>
-      <c r="C82" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A83" t="s">
-        <v>132</v>
-      </c>
-      <c r="B83" t="s">
-        <v>10</v>
-      </c>
-      <c r="C83" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A84" t="s">
-        <v>133</v>
-      </c>
-      <c r="B84" t="s">
-        <v>7</v>
-      </c>
-      <c r="C84" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A85" t="s">
-        <v>134</v>
-      </c>
-      <c r="B85" t="s">
-        <v>135</v>
-      </c>
-      <c r="C85" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A86" t="s">
-        <v>58</v>
-      </c>
-      <c r="B86" t="s">
-        <v>59</v>
-      </c>
-      <c r="C86" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A87" t="s">
-        <v>61</v>
-      </c>
-      <c r="B87" t="s">
-        <v>62</v>
-      </c>
-      <c r="C87" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A88" t="s">
-        <v>63</v>
-      </c>
-      <c r="B88" t="s">
-        <v>64</v>
-      </c>
-      <c r="C88" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="89" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A89" t="s">
-        <v>138</v>
-      </c>
-      <c r="B89" t="s">
-        <v>139</v>
-      </c>
-      <c r="C89" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="90" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A90" t="s">
-        <v>141</v>
-      </c>
-      <c r="B90" t="s">
-        <v>4</v>
-      </c>
-      <c r="C90" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A91" t="s">
-        <v>143</v>
-      </c>
-      <c r="B91" t="s">
-        <v>4</v>
-      </c>
-      <c r="C91" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A92" t="s">
-        <v>145</v>
-      </c>
-      <c r="B92" t="s">
-        <v>4</v>
-      </c>
-      <c r="C92" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="93" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A93" t="s">
-        <v>138</v>
-      </c>
-      <c r="B93" t="s">
-        <v>7</v>
-      </c>
-      <c r="C93" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="94" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A94" t="s">
-        <v>141</v>
-      </c>
-      <c r="B94" t="s">
-        <v>4</v>
-      </c>
-      <c r="C94" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A95" t="s">
-        <v>143</v>
-      </c>
-      <c r="B95" t="s">
-        <v>4</v>
-      </c>
-      <c r="C95" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="96" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A96" t="s">
-        <v>145</v>
-      </c>
-      <c r="B96" t="s">
-        <v>4</v>
-      </c>
-      <c r="C96" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="97" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A97" t="s">
-        <v>147</v>
-      </c>
-      <c r="B97" t="s">
-        <v>4</v>
-      </c>
-      <c r="C97" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="98" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A98" t="s">
-        <v>131</v>
-      </c>
-      <c r="B98" t="s">
-        <v>7</v>
-      </c>
-      <c r="C98" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="99" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A99" t="s">
-        <v>132</v>
-      </c>
-      <c r="B99" t="s">
-        <v>10</v>
-      </c>
-      <c r="C99" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="100" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A100" t="s">
-        <v>134</v>
-      </c>
-      <c r="B100" t="s">
-        <v>135</v>
-      </c>
-      <c r="C100" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="101" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A101" t="s">
-        <v>58</v>
-      </c>
-      <c r="B101" t="s">
-        <v>59</v>
-      </c>
-      <c r="C101" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="102" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A102" t="s">
-        <v>61</v>
-      </c>
-      <c r="B102" t="s">
-        <v>62</v>
-      </c>
-      <c r="C102" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="103" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A103" t="s">
-        <v>63</v>
-      </c>
-      <c r="B103" t="s">
-        <v>64</v>
-      </c>
-      <c r="C103" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="104" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A104" t="s">
-        <v>148</v>
-      </c>
-      <c r="B104" t="s">
-        <v>149</v>
-      </c>
-      <c r="C104" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="105" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A105" t="s">
-        <v>141</v>
-      </c>
-      <c r="B105" t="s">
-        <v>4</v>
-      </c>
-      <c r="C105" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="106" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A106" t="s">
-        <v>143</v>
-      </c>
-      <c r="B106" t="s">
-        <v>4</v>
-      </c>
-      <c r="C106" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="107" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A107" t="s">
-        <v>145</v>
-      </c>
-      <c r="B107" t="s">
-        <v>4</v>
-      </c>
-      <c r="C107" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="108" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A108" t="s">
-        <v>148</v>
-      </c>
-      <c r="B108" t="s">
-        <v>24</v>
-      </c>
-      <c r="C108" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="109" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A109" t="s">
-        <v>141</v>
-      </c>
-      <c r="B109" t="s">
-        <v>4</v>
-      </c>
-      <c r="C109" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="110" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A110" t="s">
-        <v>143</v>
-      </c>
-      <c r="B110" t="s">
-        <v>4</v>
-      </c>
-      <c r="C110" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="111" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A111" t="s">
-        <v>145</v>
-      </c>
-      <c r="B111" t="s">
-        <v>4</v>
-      </c>
-      <c r="C111" t="s">
-        <v>4</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:C111" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:J56" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A88CF65E-54BC-4026-8A23-04F703536EE1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{351DA637-C1A7-4EF3-822B-8B2DB036CBA2}">
   <dimension ref="A1:AA55"/>
   <sheetFormatPr defaultColWidth="8" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3807,7 +2959,7 @@
   <sheetData>
     <row r="1" spans="1:27" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>151</v>
+        <v>75</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3826,7 +2978,7 @@
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
-        <v>152</v>
+        <v>76</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3858,7 +3010,7 @@
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
-        <v>153</v>
+        <v>77</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -3871,16 +3023,16 @@
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>154</v>
+        <v>78</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>155</v>
+        <v>79</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="6" t="s">
-        <v>156</v>
+        <v>80</v>
       </c>
       <c r="G5" s="9"/>
       <c r="H5" s="9"/>
@@ -3888,14 +3040,14 @@
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>157</v>
+        <v>81</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="6" t="s">
-        <v>158</v>
+        <v>82</v>
       </c>
       <c r="G6" s="9"/>
       <c r="H6" s="9"/>
@@ -3903,24 +3055,24 @@
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
-        <v>159</v>
+        <v>83</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="6" t="s">
-        <v>160</v>
+        <v>84</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>161</v>
+        <v>85</v>
       </c>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
-        <v>162</v>
+        <v>86</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -3948,10 +3100,10 @@
     </row>
     <row r="10" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="12" t="s">
-        <v>163</v>
+        <v>87</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>164</v>
+        <v>88</v>
       </c>
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
@@ -3963,31 +3115,31 @@
     </row>
     <row r="11" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="15" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>165</v>
+        <v>89</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>166</v>
+        <v>90</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>167</v>
+        <v>91</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>168</v>
+        <v>92</v>
       </c>
       <c r="G11" s="15" t="s">
-        <v>169</v>
+        <v>93</v>
       </c>
       <c r="H11" s="15" t="s">
-        <v>170</v>
+        <v>94</v>
       </c>
       <c r="I11" s="15" t="s">
-        <v>171</v>
+        <v>95</v>
       </c>
       <c r="J11" s="15"/>
       <c r="K11" s="15"/>
@@ -4018,7 +3170,7 @@
         <v>0</v>
       </c>
       <c r="P12" s="20" t="s">
-        <v>172</v>
+        <v>96</v>
       </c>
       <c r="Q12" s="21"/>
       <c r="R12" s="21"/>
@@ -4053,23 +3205,23 @@
         <v>0</v>
       </c>
       <c r="P13" s="23" t="s">
-        <v>173</v>
+        <v>97</v>
       </c>
       <c r="Q13" s="24" t="s">
-        <v>174</v>
+        <v>98</v>
       </c>
       <c r="R13" s="24"/>
       <c r="S13" s="24"/>
       <c r="T13" s="25" t="s">
-        <v>175</v>
+        <v>99</v>
       </c>
       <c r="U13" s="25" t="s">
-        <v>176</v>
+        <v>100</v>
       </c>
       <c r="V13" s="25"/>
       <c r="W13" s="26"/>
       <c r="X13" s="27" t="s">
-        <v>177</v>
+        <v>101</v>
       </c>
     </row>
     <row r="14" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -4165,7 +3317,7 @@
         <v>50</v>
       </c>
       <c r="Y15" s="39" t="s">
-        <v>178</v>
+        <v>102</v>
       </c>
       <c r="Z15" s="40"/>
       <c r="AA15" s="40"/>
@@ -4356,7 +3508,7 @@
         <v>0</v>
       </c>
       <c r="P19" s="52" t="s">
-        <v>179</v>
+        <v>103</v>
       </c>
       <c r="Q19" s="53"/>
       <c r="R19" s="53"/>
@@ -4391,7 +3543,7 @@
         <v>0</v>
       </c>
       <c r="P20" s="55" t="s">
-        <v>180</v>
+        <v>104</v>
       </c>
       <c r="Q20" s="56"/>
       <c r="R20" s="56"/>
@@ -4429,14 +3581,14 @@
       <c r="Q21" s="59"/>
       <c r="R21" s="60"/>
       <c r="S21" s="61" t="s">
-        <v>173</v>
+        <v>97</v>
       </c>
       <c r="T21" s="61">
         <f>A19</f>
         <v>70</v>
       </c>
       <c r="U21" s="61" t="s">
-        <v>165</v>
+        <v>89</v>
       </c>
       <c r="V21" s="61"/>
       <c r="W21" s="61"/>
@@ -4469,23 +3621,23 @@
         <v>0</v>
       </c>
       <c r="P22" s="46" t="s">
-        <v>181</v>
+        <v>105</v>
       </c>
       <c r="Q22" s="63" t="s">
-        <v>182</v>
+        <v>106</v>
       </c>
       <c r="R22" s="63"/>
       <c r="S22" s="63"/>
       <c r="T22" s="49" t="s">
-        <v>183</v>
+        <v>107</v>
       </c>
       <c r="U22" s="49" t="s">
-        <v>184</v>
+        <v>108</v>
       </c>
       <c r="V22" s="50"/>
       <c r="W22" s="50"/>
       <c r="X22" s="64" t="s">
-        <v>176</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.3">
@@ -4662,7 +3814,7 @@
         <v>0</v>
       </c>
       <c r="P26" s="82" t="s">
-        <v>185</v>
+        <v>109</v>
       </c>
       <c r="Q26" s="83"/>
       <c r="R26" s="83"/>
@@ -4730,7 +3882,7 @@
         <v>0</v>
       </c>
       <c r="O28" s="86" t="s">
-        <v>186</v>
+        <v>110</v>
       </c>
       <c r="P28" s="87"/>
       <c r="Q28" s="87"/>
@@ -4767,29 +3919,29 @@
         <v>0</v>
       </c>
       <c r="O29" s="89" t="s">
-        <v>173</v>
+        <v>97</v>
       </c>
       <c r="P29" s="90" t="s">
-        <v>181</v>
+        <v>105</v>
       </c>
       <c r="Q29" s="91" t="s">
-        <v>182</v>
+        <v>106</v>
       </c>
       <c r="R29" s="92"/>
       <c r="S29" s="92"/>
       <c r="T29" s="92"/>
       <c r="U29" s="93"/>
       <c r="V29" s="94" t="s">
-        <v>187</v>
+        <v>111</v>
       </c>
       <c r="W29" s="94" t="s">
-        <v>188</v>
+        <v>112</v>
       </c>
       <c r="X29" s="95" t="s">
-        <v>189</v>
+        <v>113</v>
       </c>
       <c r="Y29" s="70" t="s">
-        <v>176</v>
+        <v>100</v>
       </c>
     </row>
     <row r="30" spans="1:25" x14ac:dyDescent="0.3">
@@ -5058,7 +4210,7 @@
       </c>
       <c r="O35" s="123"/>
       <c r="P35" s="124" t="s">
-        <v>190</v>
+        <v>114</v>
       </c>
       <c r="Q35" s="124"/>
       <c r="R35" s="124"/>
@@ -5083,25 +4235,25 @@
       <c r="B37" s="126"/>
       <c r="O37" s="18"/>
       <c r="P37" s="20" t="s">
-        <v>191</v>
+        <v>115</v>
       </c>
       <c r="Q37" s="127"/>
       <c r="R37" s="128" t="s">
-        <v>192</v>
+        <v>116</v>
       </c>
       <c r="S37" s="129" t="s">
-        <v>176</v>
+        <v>100</v>
       </c>
     </row>
     <row r="38" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="130" t="s">
-        <v>193</v>
+        <v>117</v>
       </c>
       <c r="B38" s="130"/>
       <c r="C38" s="130"/>
       <c r="O38" s="18"/>
       <c r="P38" s="131" t="s">
-        <v>173</v>
+        <v>97</v>
       </c>
       <c r="Q38" s="132">
         <f>A33</f>
@@ -5118,10 +4270,10 @@
     </row>
     <row r="39" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A39" s="65" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="B39" s="61" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C39" s="26"/>
       <c r="D39" s="26"/>
@@ -5131,23 +4283,23 @@
       <c r="H39" s="26"/>
       <c r="I39" s="26"/>
       <c r="J39" s="26" t="s">
-        <v>194</v>
+        <v>118</v>
       </c>
       <c r="K39" s="135" t="s">
-        <v>195</v>
+        <v>119</v>
       </c>
       <c r="L39" s="136" t="s">
-        <v>196</v>
+        <v>120</v>
       </c>
       <c r="O39" s="18"/>
       <c r="P39" s="137" t="s">
-        <v>197</v>
+        <v>121</v>
       </c>
       <c r="Q39" s="138"/>
       <c r="R39" s="138"/>
       <c r="S39" s="139"/>
       <c r="T39" s="140" t="s">
-        <v>198</v>
+        <v>122</v>
       </c>
     </row>
     <row r="40" spans="1:25" x14ac:dyDescent="0.3">
@@ -5165,14 +4317,14 @@
         <v>0</v>
       </c>
       <c r="K40" s="8" t="s">
-        <v>199</v>
+        <v>123</v>
       </c>
       <c r="L40" s="143" t="str">
         <f>IF(J40&lt;=5,"Pass","Fail")</f>
         <v>Pass</v>
       </c>
       <c r="M40" t="s">
-        <v>200</v>
+        <v>124</v>
       </c>
       <c r="P40" s="137"/>
       <c r="Q40" s="138"/>
@@ -5194,14 +4346,14 @@
         <v>0</v>
       </c>
       <c r="K41" s="31" t="s">
-        <v>201</v>
+        <v>125</v>
       </c>
       <c r="L41" s="148" t="str">
         <f>IF(J41&lt;=10, "Pass", "Fail")</f>
         <v>Pass</v>
       </c>
       <c r="M41" t="s">
-        <v>202</v>
+        <v>126</v>
       </c>
       <c r="P41" s="149"/>
       <c r="Q41" s="150"/>
@@ -5220,16 +4372,16 @@
     </row>
     <row r="44" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A44" s="65" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="B44" s="61" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C44" s="152" t="s">
-        <v>203</v>
+        <v>127</v>
       </c>
       <c r="D44" s="25" t="s">
-        <v>103</v>
+        <v>54</v>
       </c>
       <c r="E44" s="25"/>
       <c r="F44" s="153"/>
@@ -5244,14 +4396,14 @@
       <c r="A45" s="144"/>
       <c r="B45" s="145"/>
       <c r="C45" s="155" t="s">
-        <v>204</v>
+        <v>128</v>
       </c>
       <c r="D45" s="30">
         <v>180</v>
       </c>
       <c r="E45" s="30"/>
       <c r="F45" s="156" t="s">
-        <v>205</v>
+        <v>129</v>
       </c>
       <c r="G45" s="157"/>
       <c r="H45" s="157"/>
@@ -5262,44 +4414,44 @@
     </row>
     <row r="46" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A46" s="159" t="s">
-        <v>206</v>
+        <v>58</v>
       </c>
       <c r="B46" s="160" t="s">
-        <v>207</v>
+        <v>130</v>
       </c>
       <c r="C46" s="160"/>
       <c r="D46" s="160"/>
       <c r="E46" s="160"/>
       <c r="F46" s="160"/>
       <c r="G46" s="161" t="s">
-        <v>208</v>
+        <v>131</v>
       </c>
       <c r="H46" s="161"/>
       <c r="I46" s="98" t="s">
-        <v>209</v>
+        <v>132</v>
       </c>
       <c r="J46" s="100"/>
       <c r="K46" s="75" t="s">
-        <v>176</v>
+        <v>100</v>
       </c>
       <c r="O46" s="18"/>
     </row>
     <row r="47" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="162"/>
       <c r="B47" s="29" t="s">
-        <v>210</v>
+        <v>133</v>
       </c>
       <c r="C47" s="29" t="s">
-        <v>211</v>
+        <v>134</v>
       </c>
       <c r="D47" s="29" t="s">
-        <v>212</v>
+        <v>135</v>
       </c>
       <c r="E47" s="29" t="s">
-        <v>213</v>
+        <v>136</v>
       </c>
       <c r="F47" s="163" t="s">
-        <v>214</v>
+        <v>137</v>
       </c>
       <c r="G47" s="164"/>
       <c r="H47" s="164"/>
@@ -5310,7 +4462,7 @@
     </row>
     <row r="48" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A48" s="165" t="s">
-        <v>215</v>
+        <v>64</v>
       </c>
       <c r="B48" s="166"/>
       <c r="C48" s="166"/>
@@ -5335,7 +4487,7 @@
     </row>
     <row r="49" spans="1:15" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A49" s="50" t="s">
-        <v>216</v>
+        <v>65</v>
       </c>
       <c r="B49" s="168"/>
       <c r="C49" s="168"/>
@@ -5360,7 +4512,7 @@
     </row>
     <row r="50" spans="1:15" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A50" s="169" t="s">
-        <v>217</v>
+        <v>138</v>
       </c>
       <c r="B50" s="170"/>
       <c r="C50" s="170"/>
@@ -5383,24 +4535,24 @@
       <c r="C53" s="50"/>
       <c r="D53" s="50"/>
       <c r="E53" s="172" t="s">
-        <v>196</v>
+        <v>120</v>
       </c>
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A54" s="173" t="s">
-        <v>218</v>
+        <v>139</v>
       </c>
       <c r="B54" s="26"/>
       <c r="C54" s="174"/>
       <c r="D54" s="26" t="s">
-        <v>219</v>
+        <v>140</v>
       </c>
       <c r="E54" s="175" t="str">
         <f>IF(C54&lt;=3, "Pass", "Fail")</f>
         <v>Pass</v>
       </c>
       <c r="F54" s="8" t="s">
-        <v>220</v>
+        <v>141</v>
       </c>
       <c r="G54" s="8"/>
       <c r="H54" s="8"/>
@@ -5408,19 +4560,19 @@
     </row>
     <row r="55" spans="1:15" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A55" s="176" t="s">
-        <v>221</v>
+        <v>142</v>
       </c>
       <c r="B55" s="31"/>
       <c r="C55" s="177"/>
       <c r="D55" s="31" t="s">
-        <v>222</v>
+        <v>143</v>
       </c>
       <c r="E55" s="178" t="str">
         <f>IF(C55&gt;=1.5, "Pass", "Fail")</f>
         <v>Fail</v>
       </c>
       <c r="F55" s="8" t="s">
-        <v>223</v>
+        <v>144</v>
       </c>
       <c r="G55" s="8"/>
       <c r="H55" s="8"/>

</xml_diff>

<commit_message>
changes at Radiography portable
</commit_message>
<xml_diff>
--- a/public/templates/CArm_Template.xlsx
+++ b/public/templates/CArm_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROJECTS\anteso\anteso-frontend\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65A38083-41F4-4CA5-8E79-368AAB1652AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73315515-3FE4-4DBD-8E97-BBEB95EC2035}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Data" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="144">
   <si>
     <t>TEST: ACCURACY OF IRRADIATION TIME</t>
   </si>
@@ -2644,9 +2644,6 @@
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>8</v>
-      </c>
       <c r="B32" t="s">
         <v>8</v>
       </c>
@@ -2971,7 +2968,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:J10 A16:J20 D11:J13 A29:J62 H23:J23 A24:J24 H22:J22 A21:D21 H21:J21" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:J10 A16:J20 D11:J13 A29:J31 H23:J23 A24:J24 H22:J22 A21:D21 H21:J21 A33:J62 B32:J32" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
mammography machine kv tets fixed
</commit_message>
<xml_diff>
--- a/public/templates/CArm_Template.xlsx
+++ b/public/templates/CArm_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROJECTS\anteso\anteso-frontend\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73315515-3FE4-4DBD-8E97-BBEB95EC2035}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F60E6D-9154-46F6-A23B-00BB94B674BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Data" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="142">
   <si>
     <t>TEST: ACCURACY OF IRRADIATION TIME</t>
   </si>
@@ -98,9 +98,6 @@
     <t>TotalFiltration</t>
   </si>
   <si>
-    <t>2.5</t>
-  </si>
-  <si>
     <t>TEST: CONSISTENCY OF RADIATION OUTPUT</t>
   </si>
   <si>
@@ -216,9 +213,6 @@
   </si>
   <si>
     <t>mA Station</t>
-  </si>
-  <si>
-    <t>50</t>
   </si>
   <si>
     <t>Tolerance (CoL)</t>
@@ -1632,6 +1626,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1644,6 +1639,57 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="57" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="52" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1674,57 +1720,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="52" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1824,6 +1819,30 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1831,30 +1850,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1867,7 +1862,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2313,7 +2307,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J62"/>
+  <dimension ref="A1:J66"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="58.69921875" bestFit="1" customWidth="1"/>
@@ -2423,11 +2417,11 @@
         <f>Sheet1!P15</f>
         <v>50</v>
       </c>
-      <c r="B11" s="179">
+      <c r="B11" s="101">
         <f>Sheet1!Q15</f>
         <v>0</v>
       </c>
-      <c r="C11" s="179">
+      <c r="C11" s="101">
         <f>Sheet1!R15</f>
         <v>0</v>
       </c>
@@ -2443,11 +2437,11 @@
         <f>Sheet1!P16</f>
         <v>70</v>
       </c>
-      <c r="B12" s="179">
+      <c r="B12" s="101">
         <f>Sheet1!Q16</f>
         <v>0</v>
       </c>
-      <c r="C12" s="179">
+      <c r="C12" s="101">
         <f>Sheet1!R16</f>
         <v>0</v>
       </c>
@@ -2463,11 +2457,11 @@
         <f>Sheet1!P17</f>
         <v>90</v>
       </c>
-      <c r="B13" s="179">
+      <c r="B13" s="101">
         <f>Sheet1!Q17</f>
         <v>0</v>
       </c>
-      <c r="C13" s="179">
+      <c r="C13" s="101">
         <f>Sheet1!R17</f>
         <v>0</v>
       </c>
@@ -2483,11 +2477,11 @@
         <f>Sheet1!P18</f>
         <v>110</v>
       </c>
-      <c r="B14" s="179">
+      <c r="B14" s="101">
         <f>Sheet1!Q18</f>
         <v>0</v>
       </c>
-      <c r="C14" s="179">
+      <c r="C14" s="101">
         <f>Sheet1!R18</f>
         <v>0</v>
       </c>
@@ -2513,27 +2507,29 @@
       <c r="B17" t="s">
         <v>8</v>
       </c>
-      <c r="C17" t="s">
-        <v>25</v>
-      </c>
-      <c r="D17" t="s">
-        <v>4</v>
+      <c r="C17" s="101">
+        <f>Sheet1!R38</f>
+        <v>0</v>
+      </c>
+      <c r="D17">
+        <f>Sheet1!Q38</f>
+        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B20" t="s">
         <v>2</v>
       </c>
       <c r="C20" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D20" t="s">
         <v>2</v>
@@ -2547,19 +2543,19 @@
         <v>5</v>
       </c>
       <c r="C21" t="s">
+        <v>28</v>
+      </c>
+      <c r="D21" t="s">
         <v>29</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>30</v>
       </c>
-      <c r="E21" t="s">
-        <v>31</v>
-      </c>
       <c r="F21" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="G21" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
@@ -2624,186 +2620,171 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
+        <v>31</v>
+      </c>
+      <c r="B24" t="s">
         <v>32</v>
-      </c>
-      <c r="B24" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
+        <v>34</v>
+      </c>
+      <c r="B31" t="s">
         <v>35</v>
       </c>
-      <c r="B31" t="s">
-        <v>36</v>
-      </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <f>Sheet1!C54</f>
+        <v>0</v>
+      </c>
       <c r="B32" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>37</v>
-      </c>
-    </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
-        <v>39</v>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <f>Sheet1!C55</f>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>40</v>
-      </c>
-      <c r="B39" t="s">
-        <v>8</v>
-      </c>
-      <c r="C39" t="s">
-        <v>41</v>
-      </c>
-      <c r="D39" t="s">
-        <v>8</v>
-      </c>
-      <c r="E39" t="s">
-        <v>42</v>
-      </c>
-      <c r="F39" t="s">
-        <v>2</v>
+        <v>38</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>44</v>
+        <v>8</v>
       </c>
       <c r="C40" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D40" t="s">
-        <v>46</v>
+        <v>8</v>
+      </c>
+      <c r="E40" t="s">
+        <v>41</v>
+      </c>
+      <c r="F40" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
+        <v>42</v>
+      </c>
+      <c r="B41" t="s">
+        <v>43</v>
+      </c>
+      <c r="C41" t="s">
+        <v>44</v>
+      </c>
+      <c r="D41" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
         <v>2</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B42" t="s">
         <v>8</v>
       </c>
-      <c r="C41" t="s">
+      <c r="C42" t="s">
         <v>8</v>
       </c>
-      <c r="D41" t="s">
+      <c r="D42" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>48</v>
-      </c>
-      <c r="B44" t="s">
-        <v>2</v>
-      </c>
-      <c r="C44" t="s">
-        <v>3</v>
-      </c>
-      <c r="D44" t="s">
-        <v>4</v>
-      </c>
-      <c r="E44" t="s">
-        <v>5</v>
-      </c>
-      <c r="F44" t="s">
-        <v>2</v>
-      </c>
-      <c r="G44" t="s">
-        <v>49</v>
-      </c>
-      <c r="H44" t="s">
-        <v>50</v>
-      </c>
-      <c r="I44" t="s">
-        <v>51</v>
-      </c>
-      <c r="J44" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B45" t="s">
-        <v>54</v>
+        <v>2</v>
+      </c>
+      <c r="C45" t="s">
+        <v>3</v>
+      </c>
+      <c r="D45" t="s">
+        <v>4</v>
+      </c>
+      <c r="E45" t="s">
+        <v>5</v>
+      </c>
+      <c r="F45" t="s">
+        <v>2</v>
+      </c>
+      <c r="G45" t="s">
+        <v>48</v>
+      </c>
+      <c r="H45" t="s">
+        <v>49</v>
+      </c>
+      <c r="I45" t="s">
+        <v>50</v>
+      </c>
+      <c r="J45" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B46" t="s">
-        <v>56</v>
-      </c>
-      <c r="C46" t="s">
-        <v>57</v>
-      </c>
-      <c r="D46" t="s">
-        <v>58</v>
-      </c>
-      <c r="E46" t="s">
-        <v>59</v>
-      </c>
-      <c r="F46" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B47" t="s">
-        <v>8</v>
+        <v>55</v>
       </c>
       <c r="C47" t="s">
-        <v>8</v>
+        <v>56</v>
       </c>
       <c r="D47" t="s">
-        <v>8</v>
+        <v>57</v>
       </c>
       <c r="E47" t="s">
-        <v>8</v>
+        <v>58</v>
       </c>
       <c r="F47" t="s">
-        <v>8</v>
+        <v>59</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B48" t="s">
         <v>8</v>
@@ -2821,154 +2802,202 @@
         <v>8</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
-        <v>63</v>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>61</v>
+      </c>
+      <c r="B49" t="s">
+        <v>8</v>
+      </c>
+      <c r="C49" t="s">
+        <v>8</v>
+      </c>
+      <c r="D49" t="s">
+        <v>8</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>48</v>
-      </c>
-      <c r="B51" t="s">
-        <v>2</v>
-      </c>
-      <c r="C51" t="s">
-        <v>3</v>
-      </c>
-      <c r="D51" t="s">
-        <v>4</v>
-      </c>
-      <c r="E51" t="s">
-        <v>28</v>
-      </c>
-      <c r="F51" t="s">
-        <v>2</v>
+        <v>62</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="B52" t="s">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="C52" t="s">
-        <v>30</v>
-      </c>
-      <c r="D52" t="s">
-        <v>31</v>
+        <v>3</v>
+      </c>
+      <c r="D52">
+        <f>Sheet1!T21</f>
+        <v>70</v>
+      </c>
+      <c r="E52" t="s">
+        <v>27</v>
+      </c>
+      <c r="F52">
+        <f>Sheet1!X21</f>
+        <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B53" t="s">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="C53" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="D53" t="s">
-        <v>8</v>
+        <v>30</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A54" t="s">
+      <c r="A54">
+        <f>Sheet1!P23</f>
+        <v>1</v>
+      </c>
+      <c r="B54">
+        <f>Sheet1!Q23</f>
+        <v>0</v>
+      </c>
+      <c r="C54">
+        <f>Sheet1!R23</f>
+        <v>0</v>
+      </c>
+      <c r="D54">
+        <f>Sheet1!S23</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A55">
+        <f>Sheet1!P24</f>
         <v>2</v>
       </c>
-      <c r="B54" t="s">
-        <v>8</v>
-      </c>
-      <c r="C54" t="s">
-        <v>8</v>
-      </c>
-      <c r="D54" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55" t="s">
-        <v>66</v>
-      </c>
-      <c r="B55" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" t="s">
-        <v>48</v>
-      </c>
-      <c r="B58" t="s">
-        <v>2</v>
-      </c>
-      <c r="C58" t="s">
-        <v>3</v>
-      </c>
-      <c r="D58" t="s">
+      <c r="B55">
+        <f>Sheet1!Q24</f>
+        <v>0</v>
+      </c>
+      <c r="C55">
+        <f>Sheet1!R24</f>
+        <v>0</v>
+      </c>
+      <c r="D55">
+        <f>Sheet1!S24</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A56">
+        <f>Sheet1!P25</f>
         <v>4</v>
+      </c>
+      <c r="B56">
+        <f>Sheet1!Q25</f>
+        <v>0</v>
+      </c>
+      <c r="C56">
+        <f>Sheet1!S25</f>
+        <v>0</v>
+      </c>
+      <c r="D56">
+        <f>Sheet1!S25</f>
+        <v>0</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="B59" t="s">
-        <v>29</v>
-      </c>
-      <c r="C59" t="s">
-        <v>30</v>
-      </c>
-      <c r="D59" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A60" t="s">
-        <v>70</v>
-      </c>
-      <c r="B60" t="s">
-        <v>8</v>
-      </c>
-      <c r="C60" t="s">
-        <v>8</v>
-      </c>
-      <c r="D60" t="s">
-        <v>8</v>
+        <v>65</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>71</v>
-      </c>
-      <c r="B61" t="s">
-        <v>8</v>
-      </c>
-      <c r="C61" t="s">
-        <v>8</v>
-      </c>
-      <c r="D61" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>66</v>
+        <v>47</v>
       </c>
       <c r="B62" t="s">
+        <v>2</v>
+      </c>
+      <c r="C62" t="s">
+        <v>3</v>
+      </c>
+      <c r="D62" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
         <v>67</v>
+      </c>
+      <c r="B63" t="s">
+        <v>28</v>
+      </c>
+      <c r="C63" t="s">
+        <v>29</v>
+      </c>
+      <c r="D63" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>68</v>
+      </c>
+      <c r="B64" t="s">
+        <v>8</v>
+      </c>
+      <c r="C64" t="s">
+        <v>8</v>
+      </c>
+      <c r="D64" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>69</v>
+      </c>
+      <c r="B65" t="s">
+        <v>8</v>
+      </c>
+      <c r="C65" t="s">
+        <v>8</v>
+      </c>
+      <c r="D65" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>64</v>
+      </c>
+      <c r="B66" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:J10 A16:J20 D11:J13 A29:J31 H23:J23 A24:J24 H22:J22 A21:D21 H21:J21 A33:J62 B32:J32" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:J10 A16:J16 D11:J13 A29:J31 A24:J24 A21:D21 H21:J23 A35:J36 B32:J32 A18:J20 A17:B17 E17:J17 B34:J34 A38:J51 B37:J37 A59:J66 A52:C52 E52 G52:J52 A53:J53 E55:J55 E54:J54" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2991,35 +3020,35 @@
   <sheetData>
     <row r="1" spans="1:27" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="B1" s="170"/>
-      <c r="C1" s="170"/>
-      <c r="D1" s="170"/>
-      <c r="E1" s="170"/>
-      <c r="F1" s="170"/>
-      <c r="G1" s="170"/>
-      <c r="H1" s="170"/>
-      <c r="I1" s="170"/>
-      <c r="K1" s="177"/>
-      <c r="L1" s="177"/>
-      <c r="M1" s="177"/>
-      <c r="N1" s="178"/>
-      <c r="O1" s="178"/>
+        <v>70</v>
+      </c>
+      <c r="B1" s="168"/>
+      <c r="C1" s="168"/>
+      <c r="D1" s="168"/>
+      <c r="E1" s="168"/>
+      <c r="F1" s="168"/>
+      <c r="G1" s="168"/>
+      <c r="H1" s="168"/>
+      <c r="I1" s="168"/>
+      <c r="K1" s="178"/>
+      <c r="L1" s="178"/>
+      <c r="M1" s="178"/>
+      <c r="N1" s="179"/>
+      <c r="O1" s="179"/>
       <c r="P1" s="3"/>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B2" s="170"/>
-      <c r="C2" s="170"/>
-      <c r="D2" s="170"/>
-      <c r="E2" s="170"/>
-      <c r="F2" s="170"/>
-      <c r="G2" s="170"/>
-      <c r="H2" s="170"/>
-      <c r="I2" s="170"/>
+        <v>71</v>
+      </c>
+      <c r="B2" s="168"/>
+      <c r="C2" s="168"/>
+      <c r="D2" s="168"/>
+      <c r="E2" s="168"/>
+      <c r="F2" s="168"/>
+      <c r="G2" s="168"/>
+      <c r="H2" s="168"/>
+      <c r="I2" s="168"/>
       <c r="J2" s="5"/>
       <c r="K2" s="5"/>
       <c r="L2" s="5"/>
@@ -3027,14 +3056,14 @@
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A3" s="4"/>
-      <c r="B3" s="170"/>
-      <c r="C3" s="170"/>
-      <c r="D3" s="170"/>
-      <c r="E3" s="170"/>
-      <c r="F3" s="170"/>
-      <c r="G3" s="170"/>
-      <c r="H3" s="170"/>
-      <c r="I3" s="170"/>
+      <c r="B3" s="168"/>
+      <c r="C3" s="168"/>
+      <c r="D3" s="168"/>
+      <c r="E3" s="168"/>
+      <c r="F3" s="168"/>
+      <c r="G3" s="168"/>
+      <c r="H3" s="168"/>
+      <c r="I3" s="168"/>
       <c r="J3" s="5"/>
       <c r="K3" s="5"/>
       <c r="L3" s="5"/>
@@ -3042,89 +3071,89 @@
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="B4" s="170"/>
-      <c r="C4" s="170"/>
-      <c r="D4" s="170"/>
-      <c r="E4" s="170"/>
-      <c r="F4" s="170"/>
-      <c r="G4" s="170"/>
-      <c r="H4" s="170"/>
-      <c r="I4" s="170"/>
+        <v>72</v>
+      </c>
+      <c r="B4" s="168"/>
+      <c r="C4" s="168"/>
+      <c r="D4" s="168"/>
+      <c r="E4" s="168"/>
+      <c r="F4" s="168"/>
+      <c r="G4" s="168"/>
+      <c r="H4" s="168"/>
+      <c r="I4" s="168"/>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B5" s="168" t="s">
+        <v>74</v>
+      </c>
+      <c r="C5" s="168"/>
+      <c r="D5" s="168"/>
+      <c r="E5" s="168"/>
+      <c r="F5" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="B5" s="170" t="s">
-        <v>76</v>
-      </c>
-      <c r="C5" s="170"/>
-      <c r="D5" s="170"/>
-      <c r="E5" s="170"/>
-      <c r="F5" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="G5" s="176"/>
-      <c r="H5" s="176"/>
-      <c r="I5" s="176"/>
+      <c r="G5" s="177"/>
+      <c r="H5" s="177"/>
+      <c r="I5" s="177"/>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B6" s="170"/>
-      <c r="C6" s="170"/>
-      <c r="D6" s="170"/>
-      <c r="E6" s="170"/>
+        <v>76</v>
+      </c>
+      <c r="B6" s="168"/>
+      <c r="C6" s="168"/>
+      <c r="D6" s="168"/>
+      <c r="E6" s="168"/>
       <c r="F6" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="G6" s="176"/>
-      <c r="H6" s="176"/>
-      <c r="I6" s="176"/>
+        <v>77</v>
+      </c>
+      <c r="G6" s="177"/>
+      <c r="H6" s="177"/>
+      <c r="I6" s="177"/>
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B7" s="168"/>
+      <c r="C7" s="168"/>
+      <c r="D7" s="168"/>
+      <c r="E7" s="168"/>
+      <c r="F7" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="G7" s="168" t="s">
         <v>80</v>
       </c>
-      <c r="B7" s="170"/>
-      <c r="C7" s="170"/>
-      <c r="D7" s="170"/>
-      <c r="E7" s="170"/>
-      <c r="F7" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="G7" s="170" t="s">
-        <v>82</v>
-      </c>
-      <c r="H7" s="170"/>
-      <c r="I7" s="170"/>
+      <c r="H7" s="168"/>
+      <c r="I7" s="168"/>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="B8" s="170"/>
-      <c r="C8" s="170"/>
-      <c r="D8" s="170"/>
-      <c r="E8" s="170"/>
+        <v>81</v>
+      </c>
+      <c r="B8" s="168"/>
+      <c r="C8" s="168"/>
+      <c r="D8" s="168"/>
+      <c r="E8" s="168"/>
       <c r="F8" s="4"/>
-      <c r="G8" s="170"/>
-      <c r="H8" s="170"/>
-      <c r="I8" s="170"/>
+      <c r="G8" s="168"/>
+      <c r="H8" s="168"/>
+      <c r="I8" s="168"/>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
-      <c r="B9" s="171"/>
-      <c r="C9" s="171"/>
-      <c r="D9" s="171"/>
-      <c r="E9" s="171"/>
+      <c r="B9" s="169"/>
+      <c r="C9" s="169"/>
+      <c r="D9" s="169"/>
+      <c r="E9" s="169"/>
       <c r="F9" s="6"/>
-      <c r="G9" s="171"/>
-      <c r="H9" s="171"/>
-      <c r="I9" s="171"/>
+      <c r="G9" s="169"/>
+      <c r="H9" s="169"/>
+      <c r="I9" s="169"/>
       <c r="J9" s="8"/>
       <c r="K9" s="8"/>
       <c r="L9" s="8"/>
@@ -3132,18 +3161,18 @@
     </row>
     <row r="10" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="B10" s="172" t="s">
-        <v>85</v>
-      </c>
-      <c r="C10" s="172"/>
-      <c r="D10" s="172"/>
-      <c r="E10" s="172"/>
-      <c r="F10" s="172"/>
-      <c r="G10" s="172"/>
-      <c r="H10" s="172"/>
-      <c r="I10" s="173"/>
+        <v>82</v>
+      </c>
+      <c r="B10" s="170" t="s">
+        <v>83</v>
+      </c>
+      <c r="C10" s="170"/>
+      <c r="D10" s="170"/>
+      <c r="E10" s="170"/>
+      <c r="F10" s="170"/>
+      <c r="G10" s="170"/>
+      <c r="H10" s="170"/>
+      <c r="I10" s="171"/>
     </row>
     <row r="11" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
@@ -3153,25 +3182,25 @@
         <v>5</v>
       </c>
       <c r="C11" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="E11" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="F11" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="G11" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="F11" s="10" t="s">
+      <c r="H11" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="G11" s="10" t="s">
+      <c r="I11" s="10" t="s">
         <v>90</v>
-      </c>
-      <c r="H11" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="I11" s="10" t="s">
-        <v>92</v>
       </c>
       <c r="J11" s="10"/>
       <c r="K11" s="10"/>
@@ -3201,17 +3230,17 @@
         <f>ROUND(F12,4)</f>
         <v>0</v>
       </c>
-      <c r="P12" s="122" t="s">
-        <v>93</v>
-      </c>
-      <c r="Q12" s="174"/>
-      <c r="R12" s="174"/>
-      <c r="S12" s="174"/>
-      <c r="T12" s="174"/>
-      <c r="U12" s="174"/>
-      <c r="V12" s="174"/>
-      <c r="W12" s="174"/>
-      <c r="X12" s="175"/>
+      <c r="P12" s="113" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q12" s="172"/>
+      <c r="R12" s="172"/>
+      <c r="S12" s="172"/>
+      <c r="T12" s="172"/>
+      <c r="U12" s="172"/>
+      <c r="V12" s="172"/>
+      <c r="W12" s="172"/>
+      <c r="X12" s="173"/>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A13" s="11">
@@ -3236,24 +3265,24 @@
         <f t="shared" ref="M13:M35" si="1">ROUND(F13,4)</f>
         <v>0</v>
       </c>
-      <c r="P13" s="165" t="s">
+      <c r="P13" s="174" t="s">
+        <v>92</v>
+      </c>
+      <c r="Q13" s="176" t="s">
+        <v>93</v>
+      </c>
+      <c r="R13" s="176"/>
+      <c r="S13" s="176"/>
+      <c r="T13" s="122" t="s">
         <v>94</v>
       </c>
-      <c r="Q13" s="167" t="s">
+      <c r="U13" s="122" t="s">
         <v>95</v>
       </c>
-      <c r="R13" s="167"/>
-      <c r="S13" s="167"/>
-      <c r="T13" s="131" t="s">
+      <c r="V13" s="122"/>
+      <c r="W13" s="16"/>
+      <c r="X13" s="166" t="s">
         <v>96</v>
-      </c>
-      <c r="U13" s="131" t="s">
-        <v>97</v>
-      </c>
-      <c r="V13" s="131"/>
-      <c r="W13" s="16"/>
-      <c r="X13" s="168" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="14" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -3279,7 +3308,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P14" s="166"/>
+      <c r="P14" s="175"/>
       <c r="Q14" s="17">
         <v>1</v>
       </c>
@@ -3289,11 +3318,11 @@
       <c r="S14" s="17">
         <v>4</v>
       </c>
-      <c r="T14" s="105"/>
-      <c r="U14" s="105"/>
-      <c r="V14" s="105"/>
+      <c r="T14" s="123"/>
+      <c r="U14" s="123"/>
+      <c r="V14" s="123"/>
       <c r="W14" s="18"/>
-      <c r="X14" s="169"/>
+      <c r="X14" s="167"/>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A15" s="11">
@@ -3349,7 +3378,7 @@
         <v>50</v>
       </c>
       <c r="Y15" s="25" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="Z15" s="26"/>
       <c r="AA15" s="26"/>
@@ -3539,17 +3568,17 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P19" s="154" t="s">
-        <v>100</v>
-      </c>
-      <c r="Q19" s="155"/>
-      <c r="R19" s="155"/>
-      <c r="S19" s="155"/>
-      <c r="T19" s="155"/>
-      <c r="U19" s="155"/>
-      <c r="V19" s="155"/>
-      <c r="W19" s="155"/>
-      <c r="X19" s="156"/>
+      <c r="P19" s="155" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q19" s="156"/>
+      <c r="R19" s="156"/>
+      <c r="S19" s="156"/>
+      <c r="T19" s="156"/>
+      <c r="U19" s="156"/>
+      <c r="V19" s="156"/>
+      <c r="W19" s="156"/>
+      <c r="X19" s="157"/>
     </row>
     <row r="20" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="11">
@@ -3574,17 +3603,17 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P20" s="157" t="s">
-        <v>101</v>
-      </c>
-      <c r="Q20" s="158"/>
-      <c r="R20" s="158"/>
-      <c r="S20" s="158"/>
-      <c r="T20" s="158"/>
-      <c r="U20" s="158"/>
-      <c r="V20" s="158"/>
-      <c r="W20" s="158"/>
-      <c r="X20" s="159"/>
+      <c r="P20" s="158" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q20" s="159"/>
+      <c r="R20" s="159"/>
+      <c r="S20" s="159"/>
+      <c r="T20" s="159"/>
+      <c r="U20" s="159"/>
+      <c r="V20" s="159"/>
+      <c r="W20" s="159"/>
+      <c r="X20" s="160"/>
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A21" s="11">
@@ -3609,18 +3638,18 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P21" s="117"/>
-      <c r="Q21" s="118"/>
-      <c r="R21" s="160"/>
+      <c r="P21" s="108"/>
+      <c r="Q21" s="109"/>
+      <c r="R21" s="161"/>
       <c r="S21" s="15" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="T21" s="15">
         <f>A19</f>
         <v>70</v>
       </c>
       <c r="U21" s="15" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="V21" s="15"/>
       <c r="W21" s="15"/>
@@ -3653,23 +3682,23 @@
         <v>0</v>
       </c>
       <c r="P22" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="Q22" s="162" t="s">
+        <v>101</v>
+      </c>
+      <c r="R22" s="162"/>
+      <c r="S22" s="162"/>
+      <c r="T22" s="35" t="s">
         <v>102</v>
       </c>
-      <c r="Q22" s="161" t="s">
+      <c r="U22" s="35" t="s">
         <v>103</v>
-      </c>
-      <c r="R22" s="161"/>
-      <c r="S22" s="161"/>
-      <c r="T22" s="35" t="s">
-        <v>104</v>
-      </c>
-      <c r="U22" s="35" t="s">
-        <v>105</v>
       </c>
       <c r="V22" s="36"/>
       <c r="W22" s="36"/>
       <c r="X22" s="40" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.3">
@@ -3715,13 +3744,13 @@
         <f>ROUND((AVERAGE(Q23:S23)/P23),4)</f>
         <v>0</v>
       </c>
-      <c r="U23" s="162" t="e">
+      <c r="U23" s="163" t="e">
         <f>ROUND((MAX(T23:T26)-MIN(T23:T26))/(MAX(T23:T26)+MIN(T23:T26)),4)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="V23" s="38"/>
       <c r="W23" s="16"/>
-      <c r="X23" s="153" t="e">
+      <c r="X23" s="154" t="e">
         <f>IF(U23&lt;0.1,"Pass","Fail")</f>
         <v>#DIV/0!</v>
       </c>
@@ -3769,10 +3798,10 @@
         <f t="shared" ref="T24:T25" si="5">ROUND((AVERAGE(Q24:S24)/P24),4)</f>
         <v>0</v>
       </c>
-      <c r="U24" s="163"/>
+      <c r="U24" s="164"/>
       <c r="V24" s="46"/>
       <c r="W24" s="6"/>
-      <c r="X24" s="115"/>
+      <c r="X24" s="106"/>
     </row>
     <row r="25" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="11">
@@ -3817,10 +3846,10 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="U25" s="164"/>
+      <c r="U25" s="165"/>
       <c r="V25" s="50"/>
       <c r="W25" s="18"/>
-      <c r="X25" s="116"/>
+      <c r="X25" s="107"/>
     </row>
     <row r="26" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="11">
@@ -3845,17 +3874,17 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P26" s="132" t="s">
-        <v>106</v>
-      </c>
-      <c r="Q26" s="133"/>
-      <c r="R26" s="133"/>
-      <c r="S26" s="133"/>
-      <c r="T26" s="133"/>
-      <c r="U26" s="133"/>
-      <c r="V26" s="133"/>
-      <c r="W26" s="133"/>
-      <c r="X26" s="134"/>
+      <c r="P26" s="133" t="s">
+        <v>104</v>
+      </c>
+      <c r="Q26" s="134"/>
+      <c r="R26" s="134"/>
+      <c r="S26" s="134"/>
+      <c r="T26" s="134"/>
+      <c r="U26" s="134"/>
+      <c r="V26" s="134"/>
+      <c r="W26" s="134"/>
+      <c r="X26" s="135"/>
     </row>
     <row r="27" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="11">
@@ -3880,15 +3909,15 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P27" s="135"/>
-      <c r="Q27" s="135"/>
-      <c r="R27" s="135"/>
-      <c r="S27" s="135"/>
-      <c r="T27" s="135"/>
-      <c r="U27" s="135"/>
-      <c r="V27" s="135"/>
-      <c r="W27" s="135"/>
-      <c r="X27" s="135"/>
+      <c r="P27" s="136"/>
+      <c r="Q27" s="136"/>
+      <c r="R27" s="136"/>
+      <c r="S27" s="136"/>
+      <c r="T27" s="136"/>
+      <c r="U27" s="136"/>
+      <c r="V27" s="136"/>
+      <c r="W27" s="136"/>
+      <c r="X27" s="136"/>
     </row>
     <row r="28" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="11">
@@ -3913,19 +3942,19 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="O28" s="136" t="s">
-        <v>107</v>
-      </c>
-      <c r="P28" s="137"/>
-      <c r="Q28" s="137"/>
-      <c r="R28" s="137"/>
-      <c r="S28" s="137"/>
-      <c r="T28" s="137"/>
-      <c r="U28" s="137"/>
-      <c r="V28" s="137"/>
-      <c r="W28" s="137"/>
-      <c r="X28" s="137"/>
-      <c r="Y28" s="138"/>
+      <c r="O28" s="137" t="s">
+        <v>105</v>
+      </c>
+      <c r="P28" s="138"/>
+      <c r="Q28" s="138"/>
+      <c r="R28" s="138"/>
+      <c r="S28" s="138"/>
+      <c r="T28" s="138"/>
+      <c r="U28" s="138"/>
+      <c r="V28" s="138"/>
+      <c r="W28" s="138"/>
+      <c r="X28" s="138"/>
+      <c r="Y28" s="139"/>
     </row>
     <row r="29" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A29" s="11">
@@ -3950,30 +3979,30 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="O29" s="139" t="s">
-        <v>94</v>
-      </c>
-      <c r="P29" s="142" t="s">
-        <v>102</v>
-      </c>
-      <c r="Q29" s="145" t="s">
-        <v>103</v>
-      </c>
-      <c r="R29" s="146"/>
-      <c r="S29" s="146"/>
-      <c r="T29" s="146"/>
-      <c r="U29" s="147"/>
+      <c r="O29" s="140" t="s">
+        <v>92</v>
+      </c>
+      <c r="P29" s="143" t="s">
+        <v>100</v>
+      </c>
+      <c r="Q29" s="146" t="s">
+        <v>101</v>
+      </c>
+      <c r="R29" s="147"/>
+      <c r="S29" s="147"/>
+      <c r="T29" s="147"/>
+      <c r="U29" s="148"/>
       <c r="V29" s="51" t="s">
+        <v>106</v>
+      </c>
+      <c r="W29" s="51" t="s">
+        <v>107</v>
+      </c>
+      <c r="X29" s="151" t="s">
         <v>108</v>
       </c>
-      <c r="W29" s="51" t="s">
-        <v>109</v>
-      </c>
-      <c r="X29" s="150" t="s">
-        <v>110</v>
-      </c>
-      <c r="Y29" s="153" t="s">
-        <v>97</v>
+      <c r="Y29" s="154" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="30" spans="1:25" x14ac:dyDescent="0.3">
@@ -3999,17 +4028,17 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="O30" s="140"/>
-      <c r="P30" s="143"/>
-      <c r="Q30" s="111"/>
-      <c r="R30" s="148"/>
-      <c r="S30" s="148"/>
-      <c r="T30" s="148"/>
-      <c r="U30" s="112"/>
+      <c r="O30" s="141"/>
+      <c r="P30" s="144"/>
+      <c r="Q30" s="129"/>
+      <c r="R30" s="149"/>
+      <c r="S30" s="149"/>
+      <c r="T30" s="149"/>
+      <c r="U30" s="130"/>
       <c r="V30" s="30"/>
       <c r="W30" s="30"/>
-      <c r="X30" s="151"/>
-      <c r="Y30" s="115"/>
+      <c r="X30" s="152"/>
+      <c r="Y30" s="106"/>
     </row>
     <row r="31" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="11">
@@ -4034,17 +4063,17 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="O31" s="141"/>
-      <c r="P31" s="144"/>
-      <c r="Q31" s="113"/>
-      <c r="R31" s="149"/>
-      <c r="S31" s="149"/>
-      <c r="T31" s="149"/>
-      <c r="U31" s="114"/>
+      <c r="O31" s="142"/>
+      <c r="P31" s="145"/>
+      <c r="Q31" s="131"/>
+      <c r="R31" s="150"/>
+      <c r="S31" s="150"/>
+      <c r="T31" s="150"/>
+      <c r="U31" s="132"/>
       <c r="V31" s="52"/>
       <c r="W31" s="53"/>
-      <c r="X31" s="152"/>
-      <c r="Y31" s="116"/>
+      <c r="X31" s="153"/>
+      <c r="Y31" s="107"/>
     </row>
     <row r="32" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A32" s="11">
@@ -4206,16 +4235,16 @@
         <v>0</v>
       </c>
       <c r="O34" s="65"/>
-      <c r="P34" s="117"/>
-      <c r="Q34" s="118"/>
-      <c r="R34" s="118"/>
-      <c r="S34" s="118"/>
-      <c r="T34" s="118"/>
-      <c r="U34" s="118"/>
-      <c r="V34" s="118"/>
-      <c r="W34" s="118"/>
-      <c r="X34" s="118"/>
-      <c r="Y34" s="119"/>
+      <c r="P34" s="108"/>
+      <c r="Q34" s="109"/>
+      <c r="R34" s="109"/>
+      <c r="S34" s="109"/>
+      <c r="T34" s="109"/>
+      <c r="U34" s="109"/>
+      <c r="V34" s="109"/>
+      <c r="W34" s="109"/>
+      <c r="X34" s="109"/>
+      <c r="Y34" s="110"/>
     </row>
     <row r="35" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="11">
@@ -4241,18 +4270,18 @@
         <v>0</v>
       </c>
       <c r="O35" s="66"/>
-      <c r="P35" s="120" t="s">
-        <v>111</v>
-      </c>
-      <c r="Q35" s="120"/>
-      <c r="R35" s="120"/>
-      <c r="S35" s="120"/>
-      <c r="T35" s="120"/>
-      <c r="U35" s="120"/>
-      <c r="V35" s="120"/>
-      <c r="W35" s="120"/>
-      <c r="X35" s="120"/>
-      <c r="Y35" s="121"/>
+      <c r="P35" s="111" t="s">
+        <v>109</v>
+      </c>
+      <c r="Q35" s="111"/>
+      <c r="R35" s="111"/>
+      <c r="S35" s="111"/>
+      <c r="T35" s="111"/>
+      <c r="U35" s="111"/>
+      <c r="V35" s="111"/>
+      <c r="W35" s="111"/>
+      <c r="X35" s="111"/>
+      <c r="Y35" s="112"/>
     </row>
     <row r="36" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="2"/>
@@ -4266,26 +4295,26 @@
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="O37" s="13"/>
-      <c r="P37" s="122" t="s">
+      <c r="P37" s="113" t="s">
+        <v>110</v>
+      </c>
+      <c r="Q37" s="114"/>
+      <c r="R37" s="67" t="s">
+        <v>111</v>
+      </c>
+      <c r="S37" s="68" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="38" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="115" t="s">
         <v>112</v>
       </c>
-      <c r="Q37" s="123"/>
-      <c r="R37" s="67" t="s">
-        <v>113</v>
-      </c>
-      <c r="S37" s="68" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="38" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="124" t="s">
-        <v>114</v>
-      </c>
-      <c r="B38" s="124"/>
-      <c r="C38" s="124"/>
+      <c r="B38" s="115"/>
+      <c r="C38" s="115"/>
       <c r="O38" s="13"/>
       <c r="P38" s="69" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="Q38" s="70">
         <f>A33</f>
@@ -4315,23 +4344,23 @@
       <c r="H39" s="16"/>
       <c r="I39" s="16"/>
       <c r="J39" s="16" t="s">
+        <v>113</v>
+      </c>
+      <c r="K39" s="73" t="s">
+        <v>114</v>
+      </c>
+      <c r="L39" s="74" t="s">
         <v>115</v>
       </c>
-      <c r="K39" s="73" t="s">
+      <c r="O39" s="13"/>
+      <c r="P39" s="116" t="s">
         <v>116</v>
       </c>
-      <c r="L39" s="74" t="s">
+      <c r="Q39" s="117"/>
+      <c r="R39" s="117"/>
+      <c r="S39" s="118"/>
+      <c r="T39" s="75" t="s">
         <v>117</v>
-      </c>
-      <c r="O39" s="13"/>
-      <c r="P39" s="125" t="s">
-        <v>118</v>
-      </c>
-      <c r="Q39" s="126"/>
-      <c r="R39" s="126"/>
-      <c r="S39" s="127"/>
-      <c r="T39" s="75" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="40" spans="1:25" x14ac:dyDescent="0.3">
@@ -4349,19 +4378,19 @@
         <v>0</v>
       </c>
       <c r="K40" s="6" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="L40" s="77" t="str">
         <f>IF(J40&lt;=5,"Pass","Fail")</f>
         <v>Pass</v>
       </c>
       <c r="M40" t="s">
-        <v>121</v>
-      </c>
-      <c r="P40" s="125"/>
-      <c r="Q40" s="126"/>
-      <c r="R40" s="126"/>
-      <c r="S40" s="127"/>
+        <v>119</v>
+      </c>
+      <c r="P40" s="116"/>
+      <c r="Q40" s="117"/>
+      <c r="R40" s="117"/>
+      <c r="S40" s="118"/>
     </row>
     <row r="41" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="78"/>
@@ -4378,19 +4407,19 @@
         <v>0</v>
       </c>
       <c r="K41" s="18" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="L41" s="82" t="str">
         <f>IF(J41&lt;=10, "Pass", "Fail")</f>
         <v>Pass</v>
       </c>
       <c r="M41" t="s">
-        <v>123</v>
-      </c>
-      <c r="P41" s="128"/>
-      <c r="Q41" s="129"/>
-      <c r="R41" s="129"/>
-      <c r="S41" s="130"/>
+        <v>121</v>
+      </c>
+      <c r="P41" s="119"/>
+      <c r="Q41" s="120"/>
+      <c r="R41" s="120"/>
+      <c r="S41" s="121"/>
     </row>
     <row r="42" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A42" s="2"/>
@@ -4410,12 +4439,12 @@
         <v>5</v>
       </c>
       <c r="C44" s="83" t="s">
-        <v>124</v>
-      </c>
-      <c r="D44" s="131" t="s">
-        <v>51</v>
-      </c>
-      <c r="E44" s="131"/>
+        <v>122</v>
+      </c>
+      <c r="D44" s="122" t="s">
+        <v>50</v>
+      </c>
+      <c r="E44" s="122"/>
       <c r="F44" s="84"/>
       <c r="G44" s="84"/>
       <c r="H44" s="84"/>
@@ -4428,14 +4457,14 @@
       <c r="A45" s="78"/>
       <c r="B45" s="79"/>
       <c r="C45" s="86" t="s">
-        <v>125</v>
-      </c>
-      <c r="D45" s="105">
+        <v>123</v>
+      </c>
+      <c r="D45" s="123">
         <v>180</v>
       </c>
-      <c r="E45" s="105"/>
+      <c r="E45" s="123"/>
       <c r="F45" s="87" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="G45" s="88"/>
       <c r="H45" s="88"/>
@@ -4445,72 +4474,72 @@
       <c r="O45" s="13"/>
     </row>
     <row r="46" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A46" s="106" t="s">
-        <v>55</v>
-      </c>
-      <c r="B46" s="108" t="s">
+      <c r="A46" s="124" t="s">
+        <v>54</v>
+      </c>
+      <c r="B46" s="126" t="s">
+        <v>125</v>
+      </c>
+      <c r="C46" s="126"/>
+      <c r="D46" s="126"/>
+      <c r="E46" s="126"/>
+      <c r="F46" s="126"/>
+      <c r="G46" s="127" t="s">
+        <v>126</v>
+      </c>
+      <c r="H46" s="127"/>
+      <c r="I46" s="129" t="s">
         <v>127</v>
       </c>
-      <c r="C46" s="108"/>
-      <c r="D46" s="108"/>
-      <c r="E46" s="108"/>
-      <c r="F46" s="108"/>
-      <c r="G46" s="109" t="s">
+      <c r="J46" s="130"/>
+      <c r="K46" s="106" t="s">
+        <v>95</v>
+      </c>
+      <c r="O46" s="13"/>
+    </row>
+    <row r="47" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="125"/>
+      <c r="B47" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="H46" s="109"/>
-      <c r="I46" s="111" t="s">
+      <c r="C47" s="17" t="s">
         <v>129</v>
       </c>
-      <c r="J46" s="112"/>
-      <c r="K46" s="115" t="s">
-        <v>97</v>
-      </c>
-      <c r="O46" s="13"/>
-    </row>
-    <row r="47" spans="1:25" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="107"/>
-      <c r="B47" s="17" t="s">
+      <c r="D47" s="17" t="s">
         <v>130</v>
       </c>
-      <c r="C47" s="17" t="s">
+      <c r="E47" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="D47" s="17" t="s">
+      <c r="F47" s="90" t="s">
         <v>132</v>
       </c>
-      <c r="E47" s="17" t="s">
-        <v>133</v>
-      </c>
-      <c r="F47" s="90" t="s">
-        <v>134</v>
-      </c>
-      <c r="G47" s="110"/>
-      <c r="H47" s="110"/>
-      <c r="I47" s="113"/>
-      <c r="J47" s="114"/>
-      <c r="K47" s="116"/>
+      <c r="G47" s="128"/>
+      <c r="H47" s="128"/>
+      <c r="I47" s="131"/>
+      <c r="J47" s="132"/>
+      <c r="K47" s="107"/>
       <c r="O47" s="13"/>
     </row>
     <row r="48" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A48" s="91" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B48" s="92"/>
       <c r="C48" s="92"/>
       <c r="D48" s="92"/>
       <c r="E48" s="92"/>
       <c r="F48" s="92"/>
-      <c r="G48" s="101" t="e">
+      <c r="G48" s="102" t="e">
         <f>ROUND(3*MAX(B48:F48)/(B45),3)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H48" s="101"/>
-      <c r="I48" s="101" t="e">
+      <c r="H48" s="102"/>
+      <c r="I48" s="102" t="e">
         <f>ROUND((D45*MAX(B48:E48)/(60*B45*114)),3)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="J48" s="101"/>
+      <c r="J48" s="102"/>
       <c r="K48" s="23" t="e">
         <f>IF(I48&lt;=1, "Pass", "Fail")</f>
         <v>#DIV/0!</v>
@@ -4519,23 +4548,23 @@
     </row>
     <row r="49" spans="1:15" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A49" s="36" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B49" s="93"/>
       <c r="C49" s="93"/>
       <c r="D49" s="93"/>
       <c r="E49" s="93"/>
       <c r="F49" s="93"/>
-      <c r="G49" s="101" t="e">
+      <c r="G49" s="102" t="e">
         <f>ROUND(3*MAX(B49:F49)/(B45),3)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H49" s="101"/>
-      <c r="I49" s="101" t="e">
+      <c r="H49" s="102"/>
+      <c r="I49" s="102" t="e">
         <f>ROUND((D45*MAX(B49:F49)/(60*B45*114)),3)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="J49" s="101"/>
+      <c r="J49" s="102"/>
       <c r="K49" s="36" t="e">
         <f>IF(I49&lt;=1, "Pass", "Fail")</f>
         <v>#DIV/0!</v>
@@ -4543,19 +4572,19 @@
       <c r="O49" s="13"/>
     </row>
     <row r="50" spans="1:15" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="102" t="s">
-        <v>135</v>
-      </c>
-      <c r="B50" s="103"/>
-      <c r="C50" s="103"/>
-      <c r="D50" s="103"/>
-      <c r="E50" s="103"/>
-      <c r="F50" s="103"/>
-      <c r="G50" s="103"/>
-      <c r="H50" s="103"/>
-      <c r="I50" s="103"/>
-      <c r="J50" s="103"/>
-      <c r="K50" s="104"/>
+      <c r="A50" s="103" t="s">
+        <v>133</v>
+      </c>
+      <c r="B50" s="104"/>
+      <c r="C50" s="104"/>
+      <c r="D50" s="104"/>
+      <c r="E50" s="104"/>
+      <c r="F50" s="104"/>
+      <c r="G50" s="104"/>
+      <c r="H50" s="104"/>
+      <c r="I50" s="104"/>
+      <c r="J50" s="104"/>
+      <c r="K50" s="105"/>
       <c r="O50" s="13"/>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.3">
@@ -4567,24 +4596,24 @@
       <c r="C53" s="36"/>
       <c r="D53" s="36"/>
       <c r="E53" s="94" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A54" s="95" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B54" s="16"/>
       <c r="C54" s="96"/>
       <c r="D54" s="16" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E54" s="97" t="str">
         <f>IF(C54&lt;=3, "Pass", "Fail")</f>
         <v>Pass</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="G54" s="6"/>
       <c r="H54" s="6"/>
@@ -4592,19 +4621,19 @@
     </row>
     <row r="55" spans="1:15" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A55" s="98" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B55" s="18"/>
       <c r="C55" s="99"/>
       <c r="D55" s="18" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E55" s="100" t="str">
         <f>IF(C55&gt;=1.5, "Pass", "Fail")</f>
         <v>Fail</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="G55" s="6"/>
       <c r="H55" s="6"/>

</xml_diff>

<commit_message>
Update test data templates for various imaging modalities, including adjustments to measurement parameters, improved structure, and enhanced clarity. Refactor CArm template generation script to standardize header formats and improve data handling. Update CSV templates for consistency in test data representation across different modalities.
</commit_message>
<xml_diff>
--- a/public/templates/CArm_Template.xlsx
+++ b/public/templates/CArm_Template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O44"/>
+  <dimension ref="A1:O48"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -406,7 +406,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>FCD</v>
+        <v>FDD (cm)</v>
       </c>
       <c r="B2" t="str">
         <v>kV</v>
@@ -415,10 +415,10 @@
         <v>mA</v>
       </c>
       <c r="D2" t="str">
-        <v>Set Time (ms)</v>
+        <v>Set Time (sec)</v>
       </c>
       <c r="E2" t="str">
-        <v>Measured Time (ms)</v>
+        <v>Measured Time (sec)</v>
       </c>
       <c r="F2" t="str">
         <v>Tol Operator</v>
@@ -503,80 +503,86 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>mA Station</v>
+        <v>Tolerance Sign</v>
       </c>
       <c r="B8" t="str">
-        <v>Applied kV</v>
+        <v>Tolerance Value</v>
       </c>
       <c r="C8" t="str">
+        <v>TF Measured</v>
+      </c>
+      <c r="D8" t="str">
+        <v>TF Required</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Header 1</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Header 2</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Header 3</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Applied kVp</v>
+      </c>
+      <c r="I8" t="str">
         <v>Meas 1</v>
       </c>
-      <c r="D8" t="str">
+      <c r="J8" t="str">
         <v>Meas 2</v>
       </c>
-      <c r="E8" t="str">
+      <c r="K8" t="str">
         <v>Meas 3</v>
-      </c>
-      <c r="F8" t="str">
-        <v>Avg kV</v>
-      </c>
-      <c r="G8" t="str">
-        <v>Tolerance Sign</v>
-      </c>
-      <c r="H8" t="str">
-        <v>Tolerance Value</v>
-      </c>
-      <c r="I8" t="str">
-        <v>TF Measured</v>
-      </c>
-      <c r="J8" t="str">
-        <v>TF Required</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
+        <v>±</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2.0</v>
+      </c>
+      <c r="C9" t="str">
+        <v>1.2</v>
+      </c>
+      <c r="D9" t="str">
+        <v>1.5</v>
+      </c>
+      <c r="E9" t="str">
         <v>50 mA</v>
       </c>
-      <c r="B9" t="str">
-        <v>50</v>
-      </c>
-      <c r="C9" t="str">
-        <v>50.1</v>
-      </c>
-      <c r="D9" t="str">
-        <v>50.2</v>
-      </c>
-      <c r="E9" t="str">
-        <v/>
-      </c>
       <c r="F9" t="str">
-        <v/>
+        <v>100 mA</v>
       </c>
       <c r="G9" t="str">
-        <v>±</v>
+        <v>200 mA</v>
       </c>
       <c r="H9" t="str">
-        <v>2.0</v>
+        <v>60</v>
       </c>
       <c r="I9" t="str">
-        <v>1.2</v>
+        <v>60.1</v>
       </c>
       <c r="J9" t="str">
-        <v>1.5</v>
+        <v>60.2</v>
+      </c>
+      <c r="K9" t="str">
+        <v>60.0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>100 mA</v>
+        <v/>
       </c>
       <c r="B10" t="str">
-        <v>70</v>
+        <v/>
       </c>
       <c r="C10" t="str">
-        <v>70.1</v>
+        <v/>
       </c>
       <c r="D10" t="str">
-        <v>70.0</v>
+        <v/>
       </c>
       <c r="E10" t="str">
         <v/>
@@ -588,27 +594,30 @@
         <v/>
       </c>
       <c r="H10" t="str">
-        <v/>
+        <v>80</v>
       </c>
       <c r="I10" t="str">
-        <v/>
+        <v>80.1</v>
       </c>
       <c r="J10" t="str">
-        <v/>
+        <v>80.2</v>
+      </c>
+      <c r="K10" t="str">
+        <v>80.0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>100 mA</v>
+        <v/>
       </c>
       <c r="B11" t="str">
-        <v>90</v>
+        <v/>
       </c>
       <c r="C11" t="str">
-        <v>90.2</v>
+        <v/>
       </c>
       <c r="D11" t="str">
-        <v>90.1</v>
+        <v/>
       </c>
       <c r="E11" t="str">
         <v/>
@@ -620,269 +629,278 @@
         <v/>
       </c>
       <c r="H11" t="str">
-        <v/>
+        <v>100</v>
       </c>
       <c r="I11" t="str">
-        <v/>
+        <v>100.1</v>
       </c>
       <c r="J11" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>TEST: CONSISTENCY OF RADIATION OUTPUT</v>
+        <v>100.2</v>
+      </c>
+      <c r="K11" t="str">
+        <v>100.0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v/>
+      </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v>120</v>
+      </c>
+      <c r="I12" t="str">
+        <v>120.1</v>
+      </c>
+      <c r="J12" t="str">
+        <v>120.2</v>
+      </c>
+      <c r="K12" t="str">
+        <v>120.0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>FFD</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Time</v>
-      </c>
-      <c r="C14" t="str">
-        <v>Tolerance</v>
-      </c>
-      <c r="D14" t="str">
-        <v>Header 1</v>
-      </c>
-      <c r="E14" t="str">
-        <v>Header 2</v>
-      </c>
-      <c r="F14" t="str">
-        <v>Header 3</v>
-      </c>
-      <c r="G14" t="str">
-        <v>Header 4</v>
-      </c>
-      <c r="H14" t="str">
-        <v>Header 5</v>
-      </c>
-      <c r="I14" t="str">
-        <v>kV</v>
-      </c>
-      <c r="J14" t="str">
-        <v>mA</v>
-      </c>
-      <c r="K14" t="str">
-        <v>Meas 1</v>
-      </c>
-      <c r="L14" t="str">
-        <v>Meas 2</v>
-      </c>
-      <c r="M14" t="str">
-        <v>Meas 3</v>
-      </c>
-      <c r="N14" t="str">
-        <v>Meas 4</v>
-      </c>
-      <c r="O14" t="str">
-        <v>Meas 5</v>
+        <v>TEST: CONSISTENCY OF RADIATION OUTPUT</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>100</v>
+        <v>FDD (cm)</v>
       </c>
       <c r="B15" t="str">
-        <v>100</v>
+        <v>Time (s)</v>
       </c>
       <c r="C15" t="str">
-        <v>0.02</v>
+        <v>Tolerance</v>
       </c>
       <c r="D15" t="str">
+        <v>Header 1</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Header 2</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Header 3</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Header 4</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Header 5</v>
+      </c>
+      <c r="I15" t="str">
+        <v>kVp</v>
+      </c>
+      <c r="J15" t="str">
+        <v>mA</v>
+      </c>
+      <c r="K15" t="str">
         <v>Meas 1</v>
       </c>
-      <c r="E15" t="str">
+      <c r="L15" t="str">
         <v>Meas 2</v>
       </c>
-      <c r="F15" t="str">
+      <c r="M15" t="str">
         <v>Meas 3</v>
       </c>
-      <c r="G15" t="str">
+      <c r="N15" t="str">
         <v>Meas 4</v>
       </c>
-      <c r="H15" t="str">
+      <c r="O15" t="str">
         <v>Meas 5</v>
-      </c>
-      <c r="I15" t="str">
-        <v>50</v>
-      </c>
-      <c r="J15" t="str">
-        <v>2</v>
-      </c>
-      <c r="K15" t="str">
-        <v>0.10</v>
-      </c>
-      <c r="L15" t="str">
-        <v>0.11</v>
-      </c>
-      <c r="M15" t="str">
-        <v>0.10</v>
-      </c>
-      <c r="N15" t="str">
-        <v>0.09</v>
-      </c>
-      <c r="O15" t="str">
-        <v>0.10</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v/>
+        <v>100</v>
       </c>
       <c r="B16" t="str">
-        <v/>
+        <v>100</v>
       </c>
       <c r="C16" t="str">
-        <v/>
+        <v>0.02</v>
       </c>
       <c r="D16" t="str">
-        <v/>
+        <v>Meas 1</v>
       </c>
       <c r="E16" t="str">
-        <v/>
+        <v>Meas 2</v>
       </c>
       <c r="F16" t="str">
-        <v/>
+        <v>Meas 3</v>
       </c>
       <c r="G16" t="str">
-        <v/>
+        <v>Meas 4</v>
       </c>
       <c r="H16" t="str">
-        <v/>
+        <v>Meas 5</v>
       </c>
       <c r="I16" t="str">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="J16" t="str">
-        <v>4</v>
+        <v>100</v>
       </c>
       <c r="K16" t="str">
-        <v>0.20</v>
+        <v>10.5</v>
       </c>
       <c r="L16" t="str">
-        <v>0.21</v>
+        <v>10.4</v>
       </c>
       <c r="M16" t="str">
-        <v>0.20</v>
+        <v>10.6</v>
       </c>
       <c r="N16" t="str">
-        <v/>
+        <v>10.5</v>
       </c>
       <c r="O16" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>TEST: LOW CONTRAST RESOLUTION</v>
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v/>
+      </c>
+      <c r="B17" t="str">
+        <v/>
+      </c>
+      <c r="C17" t="str">
+        <v/>
+      </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+      <c r="H17" t="str">
+        <v/>
+      </c>
+      <c r="I17" t="str">
+        <v>100</v>
+      </c>
+      <c r="J17" t="str">
+        <v>100</v>
+      </c>
+      <c r="K17" t="str">
+        <v>12.1</v>
+      </c>
+      <c r="L17" t="str">
+        <v>12.0</v>
+      </c>
+      <c r="M17" t="str">
+        <v>12.2</v>
+      </c>
+      <c r="N17" t="str">
+        <v>12.1</v>
+      </c>
+      <c r="O17" t="str">
+        <v>12.0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Hole Size</v>
-      </c>
-      <c r="B19" t="str">
-        <v>Standard</v>
+        <v>TEST: LOW CONTRAST RESOLUTION</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
+        <v>Smallest Hole Size (mm)</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Recommended Standard</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
         <v>1.0</v>
       </c>
-      <c r="B20" t="str">
+      <c r="B21" t="str">
         <v>&gt;= 1.0 mm</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>TEST: HIGH CONTRAST RESOLUTION</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>lp/mm</v>
-      </c>
-      <c r="B23" t="str">
-        <v>Standard</v>
+        <v>TEST: HIGH CONTRAST RESOLUTION</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
+        <v>Measured Resolution (lp/mm)</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Recommended Standard (lp/mm)</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
         <v>2.0</v>
       </c>
-      <c r="B24" t="str">
+      <c r="B25" t="str">
         <v>&gt;= 2.0 lp/mm</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>TEST: EXPOSURE RATE AT TABLE TOP</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>AEC Tolerance</v>
-      </c>
-      <c r="B27" t="str">
-        <v>Non-AEC Tolerance</v>
-      </c>
-      <c r="C27" t="str">
-        <v>Min Focus Distance</v>
-      </c>
-      <c r="D27" t="str">
-        <v>Distance</v>
-      </c>
-      <c r="E27" t="str">
-        <v>kVp</v>
-      </c>
-      <c r="F27" t="str">
-        <v>mA</v>
-      </c>
-      <c r="G27" t="str">
-        <v>Exposure</v>
-      </c>
-      <c r="H27" t="str">
-        <v>Mode</v>
+        <v>TEST: EXPOSURE RATE AT TABLE TOP</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>10</v>
+        <v>Max Exposure (AEC Mode) (cGy/Min)</v>
       </c>
       <c r="B28" t="str">
-        <v>5</v>
+        <v>Max Exposure (Manual Mode) (cGy/Min)</v>
       </c>
       <c r="C28" t="str">
-        <v>30</v>
+        <v>Min. Focus to Tabletop Distance</v>
       </c>
       <c r="D28" t="str">
-        <v>100</v>
+        <v>Distance (cm)</v>
       </c>
       <c r="E28" t="str">
-        <v>80</v>
+        <v>Applied kV</v>
       </c>
       <c r="F28" t="str">
-        <v>100</v>
+        <v>Applied mA</v>
       </c>
       <c r="G28" t="str">
-        <v>0.5</v>
-      </c>
-      <c r="H28" t="str">
-        <v>AEC Mode</v>
+        <v>Exposure (cGy/Min)</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v/>
+        <v>10</v>
       </c>
       <c r="B29" t="str">
-        <v/>
+        <v>5</v>
       </c>
       <c r="C29" t="str">
-        <v/>
+        <v>30</v>
       </c>
       <c r="D29" t="str">
         <v>100</v>
@@ -894,363 +912,488 @@
         <v>100</v>
       </c>
       <c r="G29" t="str">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v/>
+      </c>
+      <c r="B30" t="str">
+        <v/>
+      </c>
+      <c r="C30" t="str">
+        <v/>
+      </c>
+      <c r="D30" t="str">
+        <v>100</v>
+      </c>
+      <c r="E30" t="str">
+        <v>80</v>
+      </c>
+      <c r="F30" t="str">
+        <v>100</v>
+      </c>
+      <c r="G30" t="str">
         <v>0.6</v>
-      </c>
-      <c r="H29" t="str">
-        <v>Manual Mode</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>TEST: TUBE HOUSING LEAKAGE</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>FCD</v>
-      </c>
-      <c r="B32" t="str">
-        <v>kV</v>
-      </c>
-      <c r="C32" t="str">
-        <v>mA</v>
-      </c>
-      <c r="D32" t="str">
-        <v>Time</v>
-      </c>
-      <c r="E32" t="str">
-        <v>Workload</v>
-      </c>
-      <c r="F32" t="str">
-        <v>Tol Value</v>
-      </c>
-      <c r="G32" t="str">
-        <v>Tol Operator</v>
-      </c>
-      <c r="H32" t="str">
-        <v>Location</v>
-      </c>
-      <c r="I32" t="str">
-        <v>Front</v>
-      </c>
-      <c r="J32" t="str">
-        <v>Back</v>
-      </c>
-      <c r="K32" t="str">
-        <v>Left</v>
-      </c>
-      <c r="L32" t="str">
-        <v>Right</v>
-      </c>
-      <c r="M32" t="str">
-        <v>Top</v>
+        <v>TEST: TUBE HOUSING LEAKAGE</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>100</v>
+        <v>FDD (cm)</v>
       </c>
       <c r="B33" t="str">
-        <v>80</v>
+        <v>kV</v>
       </c>
       <c r="C33" t="str">
-        <v>100</v>
+        <v>mA</v>
       </c>
       <c r="D33" t="str">
-        <v>1</v>
+        <v>Time (sec)</v>
       </c>
       <c r="E33" t="str">
-        <v>1000</v>
+        <v>Workload (mA·min/week)</v>
       </c>
       <c r="F33" t="str">
-        <v>1.0</v>
+        <v>Tol Value</v>
       </c>
       <c r="G33" t="str">
-        <v>less than or equal to</v>
+        <v>Tol Operator</v>
       </c>
       <c r="H33" t="str">
-        <v>Tube</v>
+        <v>Location</v>
       </c>
       <c r="I33" t="str">
-        <v>0.05</v>
+        <v>Front</v>
       </c>
       <c r="J33" t="str">
-        <v>0.03</v>
+        <v>Back</v>
       </c>
       <c r="K33" t="str">
-        <v>0.06</v>
+        <v>Left</v>
       </c>
       <c r="L33" t="str">
-        <v>0.04</v>
+        <v>Right</v>
       </c>
       <c r="M33" t="str">
-        <v>0.02</v>
+        <v>Top</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v/>
+        <v>100</v>
       </c>
       <c r="B34" t="str">
-        <v/>
+        <v>80</v>
       </c>
       <c r="C34" t="str">
-        <v/>
+        <v>100</v>
       </c>
       <c r="D34" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="E34" t="str">
-        <v/>
+        <v>1000</v>
       </c>
       <c r="F34" t="str">
-        <v/>
+        <v>1.0</v>
       </c>
       <c r="G34" t="str">
-        <v/>
+        <v>less than or equal to</v>
       </c>
       <c r="H34" t="str">
+        <v>Tube</v>
+      </c>
+      <c r="I34" t="str">
+        <v>0.05</v>
+      </c>
+      <c r="J34" t="str">
+        <v>0.03</v>
+      </c>
+      <c r="K34" t="str">
+        <v>0.06</v>
+      </c>
+      <c r="L34" t="str">
+        <v>0.04</v>
+      </c>
+      <c r="M34" t="str">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v/>
+      </c>
+      <c r="B35" t="str">
+        <v/>
+      </c>
+      <c r="C35" t="str">
+        <v/>
+      </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
+      <c r="F35" t="str">
+        <v/>
+      </c>
+      <c r="G35" t="str">
+        <v/>
+      </c>
+      <c r="H35" t="str">
         <v>Collimator</v>
       </c>
-      <c r="I34" t="str">
+      <c r="I35" t="str">
         <v>0.02</v>
       </c>
-      <c r="J34" t="str">
+      <c r="J35" t="str">
         <v>0.02</v>
       </c>
-      <c r="K34" t="str">
+      <c r="K35" t="str">
         <v>0.03</v>
       </c>
-      <c r="L34" t="str">
+      <c r="L35" t="str">
         <v>0.01</v>
       </c>
-      <c r="M34" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>TEST: LINEARITY OF MA LOADING</v>
+      <c r="M35" t="str">
+        <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>FCD</v>
-      </c>
-      <c r="B37" t="str">
-        <v>kV</v>
-      </c>
-      <c r="C37" t="str">
-        <v>Time</v>
-      </c>
-      <c r="D37" t="str">
-        <v>Tolerance</v>
-      </c>
-      <c r="E37" t="str">
-        <v>Header 1</v>
-      </c>
-      <c r="F37" t="str">
-        <v>Header 2</v>
-      </c>
-      <c r="G37" t="str">
-        <v>Header 3</v>
-      </c>
-      <c r="H37" t="str">
-        <v>mA</v>
-      </c>
-      <c r="I37" t="str">
-        <v>Meas 1</v>
-      </c>
-      <c r="J37" t="str">
-        <v>Meas 2</v>
-      </c>
-      <c r="K37" t="str">
-        <v>Meas 3</v>
+        <v>TEST: LINEARITY OF MA LOADING</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>100</v>
+        <v>FDD (cm)</v>
       </c>
       <c r="B38" t="str">
-        <v>70</v>
+        <v>kV</v>
       </c>
       <c r="C38" t="str">
-        <v>100</v>
+        <v>Time (sec)</v>
       </c>
       <c r="D38" t="str">
-        <v>0.1</v>
+        <v>Tolerance</v>
       </c>
       <c r="E38" t="str">
+        <v>Header 1</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Header 2</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Header 3</v>
+      </c>
+      <c r="H38" t="str">
+        <v>mA</v>
+      </c>
+      <c r="I38" t="str">
         <v>Meas 1</v>
       </c>
-      <c r="F38" t="str">
+      <c r="J38" t="str">
         <v>Meas 2</v>
       </c>
-      <c r="G38" t="str">
+      <c r="K38" t="str">
         <v>Meas 3</v>
-      </c>
-      <c r="H38" t="str">
-        <v>1</v>
-      </c>
-      <c r="I38" t="str">
-        <v>0.10</v>
-      </c>
-      <c r="J38" t="str">
-        <v>0.11</v>
-      </c>
-      <c r="K38" t="str">
-        <v>0.09</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v/>
+        <v>100</v>
       </c>
       <c r="B39" t="str">
-        <v/>
+        <v>70</v>
       </c>
       <c r="C39" t="str">
-        <v/>
+        <v>100</v>
       </c>
       <c r="D39" t="str">
-        <v/>
+        <v>0.1</v>
       </c>
       <c r="E39" t="str">
-        <v/>
+        <v>Meas 1</v>
       </c>
       <c r="F39" t="str">
-        <v/>
+        <v>Meas 2</v>
       </c>
       <c r="G39" t="str">
-        <v/>
+        <v>Meas 3</v>
       </c>
       <c r="H39" t="str">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="I39" t="str">
+        <v>0.10</v>
+      </c>
+      <c r="J39" t="str">
+        <v>0.11</v>
+      </c>
+      <c r="K39" t="str">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v/>
+      </c>
+      <c r="B40" t="str">
+        <v/>
+      </c>
+      <c r="C40" t="str">
+        <v/>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
+      <c r="F40" t="str">
+        <v/>
+      </c>
+      <c r="G40" t="str">
+        <v/>
+      </c>
+      <c r="H40" t="str">
+        <v>100</v>
+      </c>
+      <c r="I40" t="str">
         <v>0.20</v>
       </c>
-      <c r="J39" t="str">
+      <c r="J40" t="str">
         <v>0.21</v>
       </c>
-      <c r="K39" t="str">
+      <c r="K40" t="str">
         <v>0.19</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>TEST: LINEARITY OF MAS LOADING</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="str">
-        <v>FCD</v>
-      </c>
-      <c r="B42" t="str">
-        <v>kV</v>
-      </c>
-      <c r="C42" t="str">
-        <v>Tol Operator</v>
-      </c>
-      <c r="D42" t="str">
-        <v>Tol Value</v>
-      </c>
-      <c r="E42" t="str">
-        <v>Header 1</v>
-      </c>
-      <c r="F42" t="str">
-        <v>Header 2</v>
-      </c>
-      <c r="G42" t="str">
-        <v>Header 3</v>
-      </c>
-      <c r="H42" t="str">
-        <v>mAs</v>
-      </c>
-      <c r="I42" t="str">
-        <v>Meas 1</v>
-      </c>
-      <c r="J42" t="str">
-        <v>Meas 2</v>
-      </c>
-      <c r="K42" t="str">
-        <v>Meas 3</v>
+        <v/>
+      </c>
+      <c r="B41" t="str">
+        <v/>
+      </c>
+      <c r="C41" t="str">
+        <v/>
+      </c>
+      <c r="D41" t="str">
+        <v/>
+      </c>
+      <c r="E41" t="str">
+        <v/>
+      </c>
+      <c r="F41" t="str">
+        <v/>
+      </c>
+      <c r="G41" t="str">
+        <v/>
+      </c>
+      <c r="H41" t="str">
+        <v>200</v>
+      </c>
+      <c r="I41" t="str">
+        <v>0.40</v>
+      </c>
+      <c r="J41" t="str">
+        <v>0.41</v>
+      </c>
+      <c r="K41" t="str">
+        <v>0.39</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>100</v>
-      </c>
-      <c r="B43" t="str">
-        <v>80</v>
-      </c>
-      <c r="C43" t="str">
-        <v>&lt;=</v>
-      </c>
-      <c r="D43" t="str">
-        <v>0.1</v>
-      </c>
-      <c r="E43" t="str">
-        <v>Meas 1</v>
-      </c>
-      <c r="F43" t="str">
-        <v>Meas 2</v>
-      </c>
-      <c r="G43" t="str">
-        <v>Meas 3</v>
-      </c>
-      <c r="H43" t="str">
-        <v>5</v>
-      </c>
-      <c r="I43" t="str">
-        <v>0.10</v>
-      </c>
-      <c r="J43" t="str">
-        <v>0.11</v>
-      </c>
-      <c r="K43" t="str">
-        <v>0.09</v>
+        <v>TEST: LINEARITY OF MAS LOADING</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v/>
+        <v>FDD (cm)</v>
       </c>
       <c r="B44" t="str">
-        <v/>
+        <v>kV</v>
       </c>
       <c r="C44" t="str">
-        <v/>
+        <v>Tol Operator</v>
       </c>
       <c r="D44" t="str">
-        <v/>
+        <v>Tol Value</v>
       </c>
       <c r="E44" t="str">
-        <v/>
+        <v>Header 1</v>
       </c>
       <c r="F44" t="str">
-        <v/>
+        <v>Header 2</v>
       </c>
       <c r="G44" t="str">
-        <v/>
+        <v>Header 3</v>
       </c>
       <c r="H44" t="str">
-        <v>10</v>
+        <v>mAs Range</v>
       </c>
       <c r="I44" t="str">
-        <v>0.20</v>
+        <v>Meas 1</v>
       </c>
       <c r="J44" t="str">
-        <v>0.21</v>
+        <v>Meas 2</v>
       </c>
       <c r="K44" t="str">
-        <v>0.19</v>
+        <v>Meas 3</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>100</v>
+      </c>
+      <c r="B45" t="str">
+        <v>80</v>
+      </c>
+      <c r="C45" t="str">
+        <v>&lt;</v>
+      </c>
+      <c r="D45" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Meas 1</v>
+      </c>
+      <c r="F45" t="str">
+        <v>Meas 2</v>
+      </c>
+      <c r="G45" t="str">
+        <v>Meas 3</v>
+      </c>
+      <c r="H45" t="str">
+        <v>5 - 10</v>
+      </c>
+      <c r="I45" t="str">
+        <v>0.50</v>
+      </c>
+      <c r="J45" t="str">
+        <v>0.51</v>
+      </c>
+      <c r="K45" t="str">
+        <v>0.49</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v/>
+      </c>
+      <c r="B46" t="str">
+        <v/>
+      </c>
+      <c r="C46" t="str">
+        <v/>
+      </c>
+      <c r="D46" t="str">
+        <v/>
+      </c>
+      <c r="E46" t="str">
+        <v/>
+      </c>
+      <c r="F46" t="str">
+        <v/>
+      </c>
+      <c r="G46" t="str">
+        <v/>
+      </c>
+      <c r="H46" t="str">
+        <v>10 - 20</v>
+      </c>
+      <c r="I46" t="str">
+        <v>1.00</v>
+      </c>
+      <c r="J46" t="str">
+        <v>1.01</v>
+      </c>
+      <c r="K46" t="str">
+        <v>0.99</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v/>
+      </c>
+      <c r="B47" t="str">
+        <v/>
+      </c>
+      <c r="C47" t="str">
+        <v/>
+      </c>
+      <c r="D47" t="str">
+        <v/>
+      </c>
+      <c r="E47" t="str">
+        <v/>
+      </c>
+      <c r="F47" t="str">
+        <v/>
+      </c>
+      <c r="G47" t="str">
+        <v/>
+      </c>
+      <c r="H47" t="str">
+        <v>20 - 50</v>
+      </c>
+      <c r="I47" t="str">
+        <v>2.50</v>
+      </c>
+      <c r="J47" t="str">
+        <v>2.51</v>
+      </c>
+      <c r="K47" t="str">
+        <v>2.49</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v/>
+      </c>
+      <c r="B48" t="str">
+        <v/>
+      </c>
+      <c r="C48" t="str">
+        <v/>
+      </c>
+      <c r="D48" t="str">
+        <v/>
+      </c>
+      <c r="E48" t="str">
+        <v/>
+      </c>
+      <c r="F48" t="str">
+        <v/>
+      </c>
+      <c r="G48" t="str">
+        <v/>
+      </c>
+      <c r="H48" t="str">
+        <v>50 - 100</v>
+      </c>
+      <c r="I48" t="str">
+        <v>5.00</v>
+      </c>
+      <c r="J48" t="str">
+        <v>5.01</v>
+      </c>
+      <c r="K48" t="str">
+        <v>4.99</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O44"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O48"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update test data templates for radiography and C-Arm modalities
- Enhanced the FixedRadioFluro and Radiography templates by restructuring test sections for clarity and consistency.
- Updated measurement parameters, including adjustments to observed shifts and tolerance values, ensuring accurate data representation.
- Refactored the C-Arm template generation script to streamline the creation of Excel files, improving data handling and organization.
- Improved the accuracy of irradiation time and output consistency sections across templates, enhancing overall reporting quality.
</commit_message>
<xml_diff>
--- a/public/templates/CArm_Template.xlsx
+++ b/public/templates/CArm_Template.xlsx
@@ -3,7 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Test Data" sheetId="1" r:id="rId1"/>
+    <sheet name="With Timer" sheetId="1" r:id="rId1"/>
+    <sheet name="Without Timer" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +398,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O48"/>
+  <dimension ref="A1:M54"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="18.83203125" customWidth="1"/>
+    <col min="12" max="12" width="18.83203125" customWidth="1"/>
+    <col min="13" max="13" width="18.83203125" customWidth="1"/>
+    <col min="14" max="14" width="18.83203125" customWidth="1"/>
+    <col min="15" max="15" width="18.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -500,83 +519,104 @@
       <c r="A7" t="str">
         <v>TEST: TOTAL FILTRATION</v>
       </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
         <v>Tolerance Sign</v>
       </c>
       <c r="B8" t="str">
-        <v>Tolerance Value</v>
+        <v>±</v>
       </c>
       <c r="C8" t="str">
-        <v>TF Measured</v>
+        <v/>
       </c>
       <c r="D8" t="str">
-        <v>TF Required</v>
+        <v/>
       </c>
       <c r="E8" t="str">
-        <v>Header 1</v>
+        <v/>
       </c>
       <c r="F8" t="str">
-        <v>Header 2</v>
+        <v/>
       </c>
       <c r="G8" t="str">
-        <v>Header 3</v>
+        <v/>
       </c>
       <c r="H8" t="str">
-        <v>Applied kVp</v>
+        <v/>
       </c>
       <c r="I8" t="str">
-        <v>Meas 1</v>
+        <v/>
       </c>
       <c r="J8" t="str">
-        <v>Meas 2</v>
-      </c>
-      <c r="K8" t="str">
-        <v>Meas 3</v>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>±</v>
+        <v>Tolerance Value (kVp)</v>
       </c>
       <c r="B9" t="str">
         <v>2.0</v>
       </c>
       <c r="C9" t="str">
-        <v>1.2</v>
+        <v/>
       </c>
       <c r="D9" t="str">
-        <v>1.5</v>
+        <v/>
       </c>
       <c r="E9" t="str">
-        <v>50 mA</v>
+        <v/>
       </c>
       <c r="F9" t="str">
-        <v>100 mA</v>
+        <v/>
       </c>
       <c r="G9" t="str">
-        <v>200 mA</v>
+        <v/>
       </c>
       <c r="H9" t="str">
-        <v>60</v>
+        <v/>
       </c>
       <c r="I9" t="str">
-        <v>60.1</v>
+        <v/>
       </c>
       <c r="J9" t="str">
-        <v>60.2</v>
-      </c>
-      <c r="K9" t="str">
-        <v>60.0</v>
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v/>
+        <v>Total Filtration Required (mm Al)</v>
       </c>
       <c r="B10" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="C10" t="str">
         <v/>
@@ -594,24 +634,21 @@
         <v/>
       </c>
       <c r="H10" t="str">
-        <v>80</v>
+        <v/>
       </c>
       <c r="I10" t="str">
-        <v>80.1</v>
+        <v/>
       </c>
       <c r="J10" t="str">
-        <v>80.2</v>
-      </c>
-      <c r="K10" t="str">
-        <v>80.0</v>
+        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v/>
+        <v>Total Filtration At kVp</v>
       </c>
       <c r="B11" t="str">
-        <v/>
+        <v>80</v>
       </c>
       <c r="C11" t="str">
         <v/>
@@ -629,24 +666,21 @@
         <v/>
       </c>
       <c r="H11" t="str">
-        <v>100</v>
+        <v/>
       </c>
       <c r="I11" t="str">
-        <v>100.1</v>
+        <v/>
       </c>
       <c r="J11" t="str">
-        <v>100.2</v>
-      </c>
-      <c r="K11" t="str">
-        <v>100.0</v>
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v/>
+        <v>mA Station 1</v>
       </c>
       <c r="B12" t="str">
-        <v/>
+        <v>50</v>
       </c>
       <c r="C12" t="str">
         <v/>
@@ -664,129 +698,155 @@
         <v/>
       </c>
       <c r="H12" t="str">
-        <v>120</v>
+        <v/>
       </c>
       <c r="I12" t="str">
-        <v>120.1</v>
+        <v/>
       </c>
       <c r="J12" t="str">
-        <v>120.2</v>
-      </c>
-      <c r="K12" t="str">
-        <v>120.0</v>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>mA Station 2</v>
+      </c>
+      <c r="B13" t="str">
+        <v>100</v>
+      </c>
+      <c r="C13" t="str">
+        <v/>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>TEST: CONSISTENCY OF RADIATION OUTPUT</v>
+        <v>mA Station 3</v>
+      </c>
+      <c r="B14" t="str">
+        <v>200</v>
+      </c>
+      <c r="C14" t="str">
+        <v/>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>FDD (cm)</v>
+        <v>Applied kVp</v>
       </c>
       <c r="B15" t="str">
-        <v>Time (s)</v>
+        <v>Measured 1</v>
       </c>
       <c r="C15" t="str">
-        <v>Tolerance</v>
+        <v>Measured 2</v>
       </c>
       <c r="D15" t="str">
-        <v>Header 1</v>
+        <v>Measured 3</v>
       </c>
       <c r="E15" t="str">
-        <v>Header 2</v>
+        <v/>
       </c>
       <c r="F15" t="str">
-        <v>Header 3</v>
+        <v/>
       </c>
       <c r="G15" t="str">
-        <v>Header 4</v>
+        <v/>
       </c>
       <c r="H15" t="str">
-        <v>Header 5</v>
+        <v/>
       </c>
       <c r="I15" t="str">
-        <v>kVp</v>
+        <v/>
       </c>
       <c r="J15" t="str">
-        <v>mA</v>
-      </c>
-      <c r="K15" t="str">
-        <v>Meas 1</v>
-      </c>
-      <c r="L15" t="str">
-        <v>Meas 2</v>
-      </c>
-      <c r="M15" t="str">
-        <v>Meas 3</v>
-      </c>
-      <c r="N15" t="str">
-        <v>Meas 4</v>
-      </c>
-      <c r="O15" t="str">
-        <v>Meas 5</v>
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="B16" t="str">
-        <v>100</v>
+        <v>60.1</v>
       </c>
       <c r="C16" t="str">
-        <v>0.02</v>
+        <v>60.2</v>
       </c>
       <c r="D16" t="str">
-        <v>Meas 1</v>
+        <v>60.0</v>
       </c>
       <c r="E16" t="str">
-        <v>Meas 2</v>
+        <v/>
       </c>
       <c r="F16" t="str">
-        <v>Meas 3</v>
+        <v/>
       </c>
       <c r="G16" t="str">
-        <v>Meas 4</v>
+        <v/>
       </c>
       <c r="H16" t="str">
-        <v>Meas 5</v>
+        <v/>
       </c>
       <c r="I16" t="str">
-        <v>80</v>
+        <v/>
       </c>
       <c r="J16" t="str">
-        <v>100</v>
-      </c>
-      <c r="K16" t="str">
-        <v>10.5</v>
-      </c>
-      <c r="L16" t="str">
-        <v>10.4</v>
-      </c>
-      <c r="M16" t="str">
-        <v>10.6</v>
-      </c>
-      <c r="N16" t="str">
-        <v>10.5</v>
-      </c>
-      <c r="O16" t="str">
-        <v>10.5</v>
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v/>
+        <v>80</v>
       </c>
       <c r="B17" t="str">
-        <v/>
+        <v>80.1</v>
       </c>
       <c r="C17" t="str">
-        <v/>
+        <v>80.2</v>
       </c>
       <c r="D17" t="str">
-        <v/>
+        <v>80.0</v>
       </c>
       <c r="E17" t="str">
         <v/>
@@ -801,384 +861,1716 @@
         <v/>
       </c>
       <c r="I17" t="str">
-        <v>100</v>
+        <v/>
       </c>
       <c r="J17" t="str">
-        <v>100</v>
-      </c>
-      <c r="K17" t="str">
-        <v>12.1</v>
-      </c>
-      <c r="L17" t="str">
-        <v>12.0</v>
-      </c>
-      <c r="M17" t="str">
-        <v>12.2</v>
-      </c>
-      <c r="N17" t="str">
-        <v>12.1</v>
-      </c>
-      <c r="O17" t="str">
-        <v>12.0</v>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>100</v>
+      </c>
+      <c r="B18" t="str">
+        <v>100.1</v>
+      </c>
+      <c r="C18" t="str">
+        <v>100.2</v>
+      </c>
+      <c r="D18" t="str">
+        <v>100.0</v>
+      </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18" t="str">
+        <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
+        <v>120</v>
+      </c>
+      <c r="B19" t="str">
+        <v>120.1</v>
+      </c>
+      <c r="C19" t="str">
+        <v>120.2</v>
+      </c>
+      <c r="D19" t="str">
+        <v>120.0</v>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>TEST: CONSISTENCY OF RADIATION OUTPUT</v>
+      </c>
+      <c r="B21" t="str">
+        <v/>
+      </c>
+      <c r="C21" t="str">
+        <v/>
+      </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>FDD (cm)</v>
+      </c>
+      <c r="B22" t="str">
+        <v>100</v>
+      </c>
+      <c r="C22" t="str">
+        <v/>
+      </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+      <c r="G22" t="str">
+        <v/>
+      </c>
+      <c r="H22" t="str">
+        <v/>
+      </c>
+      <c r="I22" t="str">
+        <v/>
+      </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>kVp</v>
+      </c>
+      <c r="B23" t="str">
+        <v>mAs</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Output 1</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Output 2</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Output 3</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Output 4</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Output 5</v>
+      </c>
+      <c r="H23" t="str">
+        <v/>
+      </c>
+      <c r="I23" t="str">
+        <v/>
+      </c>
+      <c r="J23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>80</v>
+      </c>
+      <c r="B24" t="str">
+        <v>100</v>
+      </c>
+      <c r="C24" t="str">
+        <v>10.5</v>
+      </c>
+      <c r="D24" t="str">
+        <v>10.4</v>
+      </c>
+      <c r="E24" t="str">
+        <v>10.6</v>
+      </c>
+      <c r="F24" t="str">
+        <v>10.5</v>
+      </c>
+      <c r="G24" t="str">
+        <v>10.5</v>
+      </c>
+      <c r="H24" t="str">
+        <v/>
+      </c>
+      <c r="I24" t="str">
+        <v/>
+      </c>
+      <c r="J24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>100</v>
+      </c>
+      <c r="B25" t="str">
+        <v>100</v>
+      </c>
+      <c r="C25" t="str">
+        <v>12.1</v>
+      </c>
+      <c r="D25" t="str">
+        <v>12.0</v>
+      </c>
+      <c r="E25" t="str">
+        <v>12.2</v>
+      </c>
+      <c r="F25" t="str">
+        <v>12.1</v>
+      </c>
+      <c r="G25" t="str">
+        <v>12.0</v>
+      </c>
+      <c r="H25" t="str">
+        <v/>
+      </c>
+      <c r="I25" t="str">
+        <v/>
+      </c>
+      <c r="J25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Tolerance Operator</v>
+      </c>
+      <c r="B26" t="str">
+        <v>&lt;=</v>
+      </c>
+      <c r="C26" t="str">
+        <v/>
+      </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
+      <c r="F26" t="str">
+        <v/>
+      </c>
+      <c r="G26" t="str">
+        <v/>
+      </c>
+      <c r="H26" t="str">
+        <v/>
+      </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
+      <c r="J26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Tolerance Value (CoV)</v>
+      </c>
+      <c r="B27" t="str">
+        <v>0.02</v>
+      </c>
+      <c r="C27" t="str">
+        <v/>
+      </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
+      <c r="H27" t="str">
+        <v/>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
         <v>TEST: LOW CONTRAST RESOLUTION</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Smallest Hole Size (mm)</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Recommended Standard</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>1.0</v>
+      </c>
+      <c r="B31" t="str">
+        <v>&gt;= 1.0 mm</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>TEST: HIGH CONTRAST RESOLUTION</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Measured Resolution (lp/mm)</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Recommended Standard (lp/mm)</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>2.0</v>
+      </c>
+      <c r="B35" t="str">
+        <v>&gt;= 2.0 lp/mm</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>TEST: EXPOSURE RATE AT TABLE TOP</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Max Exposure (AEC Mode) (cGy/Min)</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Max Exposure (Manual Mode) (cGy/Min)</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Min. Focus to Tabletop Distance</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Distance (cm)</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Applied kV</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Applied mA</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Exposure (cGy/Min)</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>10</v>
+      </c>
+      <c r="B39" t="str">
+        <v>5</v>
+      </c>
+      <c r="C39" t="str">
+        <v>30</v>
+      </c>
+      <c r="D39" t="str">
+        <v>100</v>
+      </c>
+      <c r="E39" t="str">
+        <v>80</v>
+      </c>
+      <c r="F39" t="str">
+        <v>100</v>
+      </c>
+      <c r="G39" t="str">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v/>
+      </c>
+      <c r="B40" t="str">
+        <v/>
+      </c>
+      <c r="C40" t="str">
+        <v/>
+      </c>
+      <c r="D40" t="str">
+        <v>100</v>
+      </c>
+      <c r="E40" t="str">
+        <v>80</v>
+      </c>
+      <c r="F40" t="str">
+        <v>100</v>
+      </c>
+      <c r="G40" t="str">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>TEST: TUBE HOUSING LEAKAGE</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>FDD (cm)</v>
+      </c>
+      <c r="B43" t="str">
+        <v>kV</v>
+      </c>
+      <c r="C43" t="str">
+        <v>mA</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Time (sec)</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Workload (mA·min/week)</v>
+      </c>
+      <c r="F43" t="str">
+        <v>Tol Value</v>
+      </c>
+      <c r="G43" t="str">
+        <v>Tol Operator</v>
+      </c>
+      <c r="H43" t="str">
+        <v>Location</v>
+      </c>
+      <c r="I43" t="str">
+        <v>Front</v>
+      </c>
+      <c r="J43" t="str">
+        <v>Back</v>
+      </c>
+      <c r="K43" t="str">
+        <v>Left</v>
+      </c>
+      <c r="L43" t="str">
+        <v>Right</v>
+      </c>
+      <c r="M43" t="str">
+        <v>Top</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>100</v>
+      </c>
+      <c r="B44" t="str">
+        <v>80</v>
+      </c>
+      <c r="C44" t="str">
+        <v>100</v>
+      </c>
+      <c r="D44" t="str">
+        <v>1</v>
+      </c>
+      <c r="E44" t="str">
+        <v>1000</v>
+      </c>
+      <c r="F44" t="str">
+        <v>1.0</v>
+      </c>
+      <c r="G44" t="str">
+        <v>less than or equal to</v>
+      </c>
+      <c r="H44" t="str">
+        <v>Tube</v>
+      </c>
+      <c r="I44" t="str">
+        <v>0.05</v>
+      </c>
+      <c r="J44" t="str">
+        <v>0.03</v>
+      </c>
+      <c r="K44" t="str">
+        <v>0.06</v>
+      </c>
+      <c r="L44" t="str">
+        <v>0.04</v>
+      </c>
+      <c r="M44" t="str">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v/>
+      </c>
+      <c r="B45" t="str">
+        <v/>
+      </c>
+      <c r="C45" t="str">
+        <v/>
+      </c>
+      <c r="D45" t="str">
+        <v/>
+      </c>
+      <c r="E45" t="str">
+        <v/>
+      </c>
+      <c r="F45" t="str">
+        <v/>
+      </c>
+      <c r="G45" t="str">
+        <v/>
+      </c>
+      <c r="H45" t="str">
+        <v>Collimator</v>
+      </c>
+      <c r="I45" t="str">
+        <v>0.02</v>
+      </c>
+      <c r="J45" t="str">
+        <v>0.02</v>
+      </c>
+      <c r="K45" t="str">
+        <v>0.03</v>
+      </c>
+      <c r="L45" t="str">
+        <v>0.01</v>
+      </c>
+      <c r="M45" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>TEST: LINEARITY OF MA LOADING</v>
+      </c>
+      <c r="B47" t="str">
+        <v/>
+      </c>
+      <c r="C47" t="str">
+        <v/>
+      </c>
+      <c r="D47" t="str">
+        <v/>
+      </c>
+      <c r="E47" t="str">
+        <v/>
+      </c>
+      <c r="F47" t="str">
+        <v/>
+      </c>
+      <c r="G47" t="str">
+        <v/>
+      </c>
+      <c r="H47" t="str">
+        <v/>
+      </c>
+      <c r="I47" t="str">
+        <v/>
+      </c>
+      <c r="J47" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>FDD (cm)</v>
+      </c>
+      <c r="B48" t="str">
+        <v>100</v>
+      </c>
+      <c r="C48" t="str">
+        <v>kV</v>
+      </c>
+      <c r="D48" t="str">
+        <v>80</v>
+      </c>
+      <c r="E48" t="str">
+        <v>Time (s)</v>
+      </c>
+      <c r="F48" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="G48" t="str">
+        <v/>
+      </c>
+      <c r="H48" t="str">
+        <v/>
+      </c>
+      <c r="I48" t="str">
+        <v/>
+      </c>
+      <c r="J48" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>mA Applied</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Measured Output 1</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Measured Output 2</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Measured Output 3</v>
+      </c>
+      <c r="E49" t="str">
+        <v/>
+      </c>
+      <c r="F49" t="str">
+        <v/>
+      </c>
+      <c r="G49" t="str">
+        <v/>
+      </c>
+      <c r="H49" t="str">
+        <v/>
+      </c>
+      <c r="I49" t="str">
+        <v/>
+      </c>
+      <c r="J49" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>50</v>
+      </c>
+      <c r="B50" t="str">
+        <v>0.10</v>
+      </c>
+      <c r="C50" t="str">
+        <v>0.11</v>
+      </c>
+      <c r="D50" t="str">
+        <v>0.09</v>
+      </c>
+      <c r="E50" t="str">
+        <v/>
+      </c>
+      <c r="F50" t="str">
+        <v/>
+      </c>
+      <c r="G50" t="str">
+        <v/>
+      </c>
+      <c r="H50" t="str">
+        <v/>
+      </c>
+      <c r="I50" t="str">
+        <v/>
+      </c>
+      <c r="J50" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>100</v>
+      </c>
+      <c r="B51" t="str">
+        <v>0.20</v>
+      </c>
+      <c r="C51" t="str">
+        <v>0.21</v>
+      </c>
+      <c r="D51" t="str">
+        <v>0.19</v>
+      </c>
+      <c r="E51" t="str">
+        <v/>
+      </c>
+      <c r="F51" t="str">
+        <v/>
+      </c>
+      <c r="G51" t="str">
+        <v/>
+      </c>
+      <c r="H51" t="str">
+        <v/>
+      </c>
+      <c r="I51" t="str">
+        <v/>
+      </c>
+      <c r="J51" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>200</v>
+      </c>
+      <c r="B52" t="str">
+        <v>0.40</v>
+      </c>
+      <c r="C52" t="str">
+        <v>0.41</v>
+      </c>
+      <c r="D52" t="str">
+        <v>0.39</v>
+      </c>
+      <c r="E52" t="str">
+        <v/>
+      </c>
+      <c r="F52" t="str">
+        <v/>
+      </c>
+      <c r="G52" t="str">
+        <v/>
+      </c>
+      <c r="H52" t="str">
+        <v/>
+      </c>
+      <c r="I52" t="str">
+        <v/>
+      </c>
+      <c r="J52" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Tolerance Operator</v>
+      </c>
+      <c r="B53" t="str">
+        <v>&lt;=</v>
+      </c>
+      <c r="C53" t="str">
+        <v/>
+      </c>
+      <c r="D53" t="str">
+        <v/>
+      </c>
+      <c r="E53" t="str">
+        <v/>
+      </c>
+      <c r="F53" t="str">
+        <v/>
+      </c>
+      <c r="G53" t="str">
+        <v/>
+      </c>
+      <c r="H53" t="str">
+        <v/>
+      </c>
+      <c r="I53" t="str">
+        <v/>
+      </c>
+      <c r="J53" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Tolerance Value (CoL)</v>
+      </c>
+      <c r="B54" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="C54" t="str">
+        <v/>
+      </c>
+      <c r="D54" t="str">
+        <v/>
+      </c>
+      <c r="E54" t="str">
+        <v/>
+      </c>
+      <c r="F54" t="str">
+        <v/>
+      </c>
+      <c r="G54" t="str">
+        <v/>
+      </c>
+      <c r="H54" t="str">
+        <v/>
+      </c>
+      <c r="I54" t="str">
+        <v/>
+      </c>
+      <c r="J54" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:M54"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M49"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="18.83203125" customWidth="1"/>
+    <col min="12" max="12" width="18.83203125" customWidth="1"/>
+    <col min="13" max="13" width="18.83203125" customWidth="1"/>
+    <col min="14" max="14" width="18.83203125" customWidth="1"/>
+    <col min="15" max="15" width="18.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>TEST: TOTAL FILTRATION</v>
+      </c>
+      <c r="B1" t="str">
+        <v/>
+      </c>
+      <c r="C1" t="str">
+        <v/>
+      </c>
+      <c r="D1" t="str">
+        <v/>
+      </c>
+      <c r="E1" t="str">
+        <v/>
+      </c>
+      <c r="F1" t="str">
+        <v/>
+      </c>
+      <c r="G1" t="str">
+        <v/>
+      </c>
+      <c r="H1" t="str">
+        <v/>
+      </c>
+      <c r="I1" t="str">
+        <v/>
+      </c>
+      <c r="J1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Tolerance Sign</v>
+      </c>
+      <c r="B2" t="str">
+        <v>±</v>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Tolerance Value (kVp)</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2.0</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Total Filtration Required (mm Al)</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2.5</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Total Filtration At kVp</v>
+      </c>
+      <c r="B5" t="str">
+        <v>80</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>mA Station 1</v>
+      </c>
+      <c r="B6" t="str">
+        <v>50</v>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>mA Station 2</v>
+      </c>
+      <c r="B7" t="str">
+        <v>100</v>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>mA Station 3</v>
+      </c>
+      <c r="B8" t="str">
+        <v>200</v>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Applied kVp</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Measured 1</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Measured 2</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Measured 3</v>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>60</v>
+      </c>
+      <c r="B10" t="str">
+        <v>60.1</v>
+      </c>
+      <c r="C10" t="str">
+        <v>60.2</v>
+      </c>
+      <c r="D10" t="str">
+        <v>60.0</v>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>80</v>
+      </c>
+      <c r="B11" t="str">
+        <v>80.1</v>
+      </c>
+      <c r="C11" t="str">
+        <v>80.2</v>
+      </c>
+      <c r="D11" t="str">
+        <v>80.0</v>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>100</v>
+      </c>
+      <c r="B12" t="str">
+        <v>100.1</v>
+      </c>
+      <c r="C12" t="str">
+        <v>100.2</v>
+      </c>
+      <c r="D12" t="str">
+        <v>100.0</v>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>120</v>
+      </c>
+      <c r="B13" t="str">
+        <v>120.1</v>
+      </c>
+      <c r="C13" t="str">
+        <v>120.2</v>
+      </c>
+      <c r="D13" t="str">
+        <v>120.0</v>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>TEST: CONSISTENCY OF RADIATION OUTPUT</v>
+      </c>
+      <c r="B15" t="str">
+        <v/>
+      </c>
+      <c r="C15" t="str">
+        <v/>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>FDD (cm)</v>
+      </c>
+      <c r="B16" t="str">
+        <v>100</v>
+      </c>
+      <c r="C16" t="str">
+        <v/>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>kVp</v>
+      </c>
+      <c r="B17" t="str">
+        <v>mAs</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Output 1</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Output 2</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Output 3</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Output 4</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Output 5</v>
+      </c>
+      <c r="H17" t="str">
+        <v/>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>80</v>
+      </c>
+      <c r="B18" t="str">
+        <v>100</v>
+      </c>
+      <c r="C18" t="str">
+        <v>10.5</v>
+      </c>
+      <c r="D18" t="str">
+        <v>10.4</v>
+      </c>
+      <c r="E18" t="str">
+        <v>10.6</v>
+      </c>
+      <c r="F18" t="str">
+        <v>10.5</v>
+      </c>
+      <c r="G18" t="str">
+        <v>10.5</v>
+      </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>100</v>
+      </c>
+      <c r="B19" t="str">
+        <v>100</v>
+      </c>
+      <c r="C19" t="str">
+        <v>12.1</v>
+      </c>
+      <c r="D19" t="str">
+        <v>12.0</v>
+      </c>
+      <c r="E19" t="str">
+        <v>12.2</v>
+      </c>
+      <c r="F19" t="str">
+        <v>12.1</v>
+      </c>
+      <c r="G19" t="str">
+        <v>12.0</v>
+      </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19" t="str">
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Smallest Hole Size (mm)</v>
+        <v>Tolerance Operator</v>
       </c>
       <c r="B20" t="str">
-        <v>Recommended Standard</v>
+        <v>&lt;=</v>
+      </c>
+      <c r="C20" t="str">
+        <v/>
+      </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20" t="str">
+        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>1.0</v>
+        <v>Tolerance Value (CoV)</v>
       </c>
       <c r="B21" t="str">
-        <v>&gt;= 1.0 mm</v>
+        <v>0.02</v>
+      </c>
+      <c r="C21" t="str">
+        <v/>
+      </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
+        <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>TEST: HIGH CONTRAST RESOLUTION</v>
+        <v>TEST: LOW CONTRAST RESOLUTION</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Measured Resolution (lp/mm)</v>
+        <v>Smallest Hole Size (mm)</v>
       </c>
       <c r="B24" t="str">
-        <v>Recommended Standard (lp/mm)</v>
+        <v>Recommended Standard</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="B25" t="str">
-        <v>&gt;= 2.0 lp/mm</v>
+        <v>&gt;= 1.0 mm</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>TEST: EXPOSURE RATE AT TABLE TOP</v>
+        <v>TEST: HIGH CONTRAST RESOLUTION</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Max Exposure (AEC Mode) (cGy/Min)</v>
+        <v>Measured Resolution (lp/mm)</v>
       </c>
       <c r="B28" t="str">
-        <v>Max Exposure (Manual Mode) (cGy/Min)</v>
-      </c>
-      <c r="C28" t="str">
-        <v>Min. Focus to Tabletop Distance</v>
-      </c>
-      <c r="D28" t="str">
-        <v>Distance (cm)</v>
-      </c>
-      <c r="E28" t="str">
-        <v>Applied kV</v>
-      </c>
-      <c r="F28" t="str">
-        <v>Applied mA</v>
-      </c>
-      <c r="G28" t="str">
-        <v>Exposure (cGy/Min)</v>
+        <v>Recommended Standard (lp/mm)</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>10</v>
+        <v>2.0</v>
       </c>
       <c r="B29" t="str">
-        <v>5</v>
-      </c>
-      <c r="C29" t="str">
-        <v>30</v>
-      </c>
-      <c r="D29" t="str">
-        <v>100</v>
-      </c>
-      <c r="E29" t="str">
-        <v>80</v>
-      </c>
-      <c r="F29" t="str">
-        <v>100</v>
-      </c>
-      <c r="G29" t="str">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v/>
-      </c>
-      <c r="B30" t="str">
-        <v/>
-      </c>
-      <c r="C30" t="str">
-        <v/>
-      </c>
-      <c r="D30" t="str">
-        <v>100</v>
-      </c>
-      <c r="E30" t="str">
-        <v>80</v>
-      </c>
-      <c r="F30" t="str">
-        <v>100</v>
-      </c>
-      <c r="G30" t="str">
-        <v>0.6</v>
+        <v>&gt;= 2.0 lp/mm</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>TEST: EXPOSURE RATE AT TABLE TOP</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>TEST: TUBE HOUSING LEAKAGE</v>
+        <v>Max Exposure (AEC Mode) (cGy/Min)</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Max Exposure (Manual Mode) (cGy/Min)</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Min. Focus to Tabletop Distance</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Distance (cm)</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Applied kV</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Applied mA</v>
+      </c>
+      <c r="G32" t="str">
+        <v>Exposure (cGy/Min)</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>FDD (cm)</v>
+        <v>10</v>
       </c>
       <c r="B33" t="str">
-        <v>kV</v>
+        <v>5</v>
       </c>
       <c r="C33" t="str">
-        <v>mA</v>
+        <v>30</v>
       </c>
       <c r="D33" t="str">
-        <v>Time (sec)</v>
+        <v>100</v>
       </c>
       <c r="E33" t="str">
-        <v>Workload (mA·min/week)</v>
+        <v>80</v>
       </c>
       <c r="F33" t="str">
-        <v>Tol Value</v>
+        <v>100</v>
       </c>
       <c r="G33" t="str">
-        <v>Tol Operator</v>
-      </c>
-      <c r="H33" t="str">
-        <v>Location</v>
-      </c>
-      <c r="I33" t="str">
-        <v>Front</v>
-      </c>
-      <c r="J33" t="str">
-        <v>Back</v>
-      </c>
-      <c r="K33" t="str">
-        <v>Left</v>
-      </c>
-      <c r="L33" t="str">
-        <v>Right</v>
-      </c>
-      <c r="M33" t="str">
-        <v>Top</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>100</v>
+        <v/>
       </c>
       <c r="B34" t="str">
+        <v/>
+      </c>
+      <c r="C34" t="str">
+        <v/>
+      </c>
+      <c r="D34" t="str">
+        <v>100</v>
+      </c>
+      <c r="E34" t="str">
         <v>80</v>
       </c>
-      <c r="C34" t="str">
-        <v>100</v>
-      </c>
-      <c r="D34" t="str">
-        <v>1</v>
-      </c>
-      <c r="E34" t="str">
-        <v>1000</v>
-      </c>
       <c r="F34" t="str">
-        <v>1.0</v>
+        <v>100</v>
       </c>
       <c r="G34" t="str">
-        <v>less than or equal to</v>
-      </c>
-      <c r="H34" t="str">
-        <v>Tube</v>
-      </c>
-      <c r="I34" t="str">
-        <v>0.05</v>
-      </c>
-      <c r="J34" t="str">
-        <v>0.03</v>
-      </c>
-      <c r="K34" t="str">
-        <v>0.06</v>
-      </c>
-      <c r="L34" t="str">
-        <v>0.04</v>
-      </c>
-      <c r="M34" t="str">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v/>
-      </c>
-      <c r="B35" t="str">
-        <v/>
-      </c>
-      <c r="C35" t="str">
-        <v/>
-      </c>
-      <c r="D35" t="str">
-        <v/>
-      </c>
-      <c r="E35" t="str">
-        <v/>
-      </c>
-      <c r="F35" t="str">
-        <v/>
-      </c>
-      <c r="G35" t="str">
-        <v/>
-      </c>
-      <c r="H35" t="str">
-        <v>Collimator</v>
-      </c>
-      <c r="I35" t="str">
-        <v>0.02</v>
-      </c>
-      <c r="J35" t="str">
-        <v>0.02</v>
-      </c>
-      <c r="K35" t="str">
-        <v>0.03</v>
-      </c>
-      <c r="L35" t="str">
-        <v>0.01</v>
-      </c>
-      <c r="M35" t="str">
-        <v/>
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>TEST: TUBE HOUSING LEAKAGE</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>TEST: LINEARITY OF MA LOADING</v>
+        <v>FDD (cm)</v>
+      </c>
+      <c r="B37" t="str">
+        <v>kV</v>
+      </c>
+      <c r="C37" t="str">
+        <v>mA</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Time (sec)</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Workload (mA·min/week)</v>
+      </c>
+      <c r="F37" t="str">
+        <v>Tol Value</v>
+      </c>
+      <c r="G37" t="str">
+        <v>Tol Operator</v>
+      </c>
+      <c r="H37" t="str">
+        <v>Location</v>
+      </c>
+      <c r="I37" t="str">
+        <v>Front</v>
+      </c>
+      <c r="J37" t="str">
+        <v>Back</v>
+      </c>
+      <c r="K37" t="str">
+        <v>Left</v>
+      </c>
+      <c r="L37" t="str">
+        <v>Right</v>
+      </c>
+      <c r="M37" t="str">
+        <v>Top</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>FDD (cm)</v>
+        <v>100</v>
       </c>
       <c r="B38" t="str">
-        <v>kV</v>
+        <v>80</v>
       </c>
       <c r="C38" t="str">
-        <v>Time (sec)</v>
+        <v>100</v>
       </c>
       <c r="D38" t="str">
-        <v>Tolerance</v>
+        <v>1</v>
       </c>
       <c r="E38" t="str">
-        <v>Header 1</v>
+        <v>1000</v>
       </c>
       <c r="F38" t="str">
-        <v>Header 2</v>
+        <v>1.0</v>
       </c>
       <c r="G38" t="str">
-        <v>Header 3</v>
+        <v>less than or equal to</v>
       </c>
       <c r="H38" t="str">
-        <v>mA</v>
+        <v>Tube</v>
       </c>
       <c r="I38" t="str">
-        <v>Meas 1</v>
+        <v>0.05</v>
       </c>
       <c r="J38" t="str">
-        <v>Meas 2</v>
+        <v>0.03</v>
       </c>
       <c r="K38" t="str">
-        <v>Meas 3</v>
+        <v>0.06</v>
+      </c>
+      <c r="L38" t="str">
+        <v>0.04</v>
+      </c>
+      <c r="M38" t="str">
+        <v>0.02</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>100</v>
+        <v/>
       </c>
       <c r="B39" t="str">
-        <v>70</v>
+        <v/>
       </c>
       <c r="C39" t="str">
-        <v>100</v>
+        <v/>
       </c>
       <c r="D39" t="str">
-        <v>0.1</v>
+        <v/>
       </c>
       <c r="E39" t="str">
-        <v>Meas 1</v>
+        <v/>
       </c>
       <c r="F39" t="str">
-        <v>Meas 2</v>
+        <v/>
       </c>
       <c r="G39" t="str">
-        <v>Meas 3</v>
+        <v/>
       </c>
       <c r="H39" t="str">
-        <v>50</v>
+        <v>Collimator</v>
       </c>
       <c r="I39" t="str">
-        <v>0.10</v>
+        <v>0.02</v>
       </c>
       <c r="J39" t="str">
-        <v>0.11</v>
+        <v>0.02</v>
       </c>
       <c r="K39" t="str">
-        <v>0.09</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="str">
-        <v/>
-      </c>
-      <c r="B40" t="str">
-        <v/>
-      </c>
-      <c r="C40" t="str">
-        <v/>
-      </c>
-      <c r="D40" t="str">
-        <v/>
-      </c>
-      <c r="E40" t="str">
-        <v/>
-      </c>
-      <c r="F40" t="str">
-        <v/>
-      </c>
-      <c r="G40" t="str">
-        <v/>
-      </c>
-      <c r="H40" t="str">
-        <v>100</v>
-      </c>
-      <c r="I40" t="str">
-        <v>0.20</v>
-      </c>
-      <c r="J40" t="str">
-        <v>0.21</v>
-      </c>
-      <c r="K40" t="str">
-        <v>0.19</v>
+        <v>0.03</v>
+      </c>
+      <c r="L39" t="str">
+        <v>0.01</v>
+      </c>
+      <c r="M39" t="str">
+        <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v/>
+        <v>TEST: LINEARITY OF MAS LOADING</v>
       </c>
       <c r="B41" t="str">
         <v/>
@@ -1199,105 +2591,155 @@
         <v/>
       </c>
       <c r="H41" t="str">
-        <v>200</v>
+        <v/>
       </c>
       <c r="I41" t="str">
-        <v>0.40</v>
+        <v/>
       </c>
       <c r="J41" t="str">
-        <v>0.41</v>
-      </c>
-      <c r="K41" t="str">
-        <v>0.39</v>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>FDD (cm)</v>
+      </c>
+      <c r="B42" t="str">
+        <v>100</v>
+      </c>
+      <c r="C42" t="str">
+        <v>kV</v>
+      </c>
+      <c r="D42" t="str">
+        <v>80</v>
+      </c>
+      <c r="E42" t="str">
+        <v/>
+      </c>
+      <c r="F42" t="str">
+        <v/>
+      </c>
+      <c r="G42" t="str">
+        <v/>
+      </c>
+      <c r="H42" t="str">
+        <v/>
+      </c>
+      <c r="I42" t="str">
+        <v/>
+      </c>
+      <c r="J42" t="str">
+        <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>TEST: LINEARITY OF MAS LOADING</v>
+        <v>mAs Range</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Measured Output 1</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Measured Output 2</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Measured Output 3</v>
+      </c>
+      <c r="E43" t="str">
+        <v/>
+      </c>
+      <c r="F43" t="str">
+        <v/>
+      </c>
+      <c r="G43" t="str">
+        <v/>
+      </c>
+      <c r="H43" t="str">
+        <v/>
+      </c>
+      <c r="I43" t="str">
+        <v/>
+      </c>
+      <c r="J43" t="str">
+        <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>FDD (cm)</v>
+        <v>5 - 10</v>
       </c>
       <c r="B44" t="str">
-        <v>kV</v>
+        <v>0.50</v>
       </c>
       <c r="C44" t="str">
-        <v>Tol Operator</v>
+        <v>0.51</v>
       </c>
       <c r="D44" t="str">
-        <v>Tol Value</v>
+        <v>0.49</v>
       </c>
       <c r="E44" t="str">
-        <v>Header 1</v>
+        <v/>
       </c>
       <c r="F44" t="str">
-        <v>Header 2</v>
+        <v/>
       </c>
       <c r="G44" t="str">
-        <v>Header 3</v>
+        <v/>
       </c>
       <c r="H44" t="str">
-        <v>mAs Range</v>
+        <v/>
       </c>
       <c r="I44" t="str">
-        <v>Meas 1</v>
+        <v/>
       </c>
       <c r="J44" t="str">
-        <v>Meas 2</v>
-      </c>
-      <c r="K44" t="str">
-        <v>Meas 3</v>
+        <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>100</v>
+        <v>10 - 20</v>
       </c>
       <c r="B45" t="str">
-        <v>80</v>
+        <v>1.00</v>
       </c>
       <c r="C45" t="str">
-        <v>&lt;</v>
+        <v>1.01</v>
       </c>
       <c r="D45" t="str">
-        <v>0.1</v>
+        <v>0.99</v>
       </c>
       <c r="E45" t="str">
-        <v>Meas 1</v>
+        <v/>
       </c>
       <c r="F45" t="str">
-        <v>Meas 2</v>
+        <v/>
       </c>
       <c r="G45" t="str">
-        <v>Meas 3</v>
+        <v/>
       </c>
       <c r="H45" t="str">
-        <v>5 - 10</v>
+        <v/>
       </c>
       <c r="I45" t="str">
-        <v>0.50</v>
+        <v/>
       </c>
       <c r="J45" t="str">
-        <v>0.51</v>
-      </c>
-      <c r="K45" t="str">
-        <v>0.49</v>
+        <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v/>
+        <v>20 - 50</v>
       </c>
       <c r="B46" t="str">
-        <v/>
+        <v>2.50</v>
       </c>
       <c r="C46" t="str">
-        <v/>
+        <v>2.51</v>
       </c>
       <c r="D46" t="str">
-        <v/>
+        <v>2.49</v>
       </c>
       <c r="E46" t="str">
         <v/>
@@ -1309,30 +2751,27 @@
         <v/>
       </c>
       <c r="H46" t="str">
-        <v>10 - 20</v>
+        <v/>
       </c>
       <c r="I46" t="str">
-        <v>1.00</v>
+        <v/>
       </c>
       <c r="J46" t="str">
-        <v>1.01</v>
-      </c>
-      <c r="K46" t="str">
-        <v>0.99</v>
+        <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v/>
+        <v>50 - 100</v>
       </c>
       <c r="B47" t="str">
-        <v/>
+        <v>5.00</v>
       </c>
       <c r="C47" t="str">
-        <v/>
+        <v>5.01</v>
       </c>
       <c r="D47" t="str">
-        <v/>
+        <v>4.99</v>
       </c>
       <c r="E47" t="str">
         <v/>
@@ -1344,24 +2783,21 @@
         <v/>
       </c>
       <c r="H47" t="str">
-        <v>20 - 50</v>
+        <v/>
       </c>
       <c r="I47" t="str">
-        <v>2.50</v>
+        <v/>
       </c>
       <c r="J47" t="str">
-        <v>2.51</v>
-      </c>
-      <c r="K47" t="str">
-        <v>2.49</v>
+        <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v/>
+        <v>Tolerance Operator</v>
       </c>
       <c r="B48" t="str">
-        <v/>
+        <v>&lt;=</v>
       </c>
       <c r="C48" t="str">
         <v/>
@@ -1379,21 +2815,50 @@
         <v/>
       </c>
       <c r="H48" t="str">
-        <v>50 - 100</v>
+        <v/>
       </c>
       <c r="I48" t="str">
-        <v>5.00</v>
+        <v/>
       </c>
       <c r="J48" t="str">
-        <v>5.01</v>
-      </c>
-      <c r="K48" t="str">
-        <v>4.99</v>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Tolerance Value (CoL)</v>
+      </c>
+      <c r="B49" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="C49" t="str">
+        <v/>
+      </c>
+      <c r="D49" t="str">
+        <v/>
+      </c>
+      <c r="E49" t="str">
+        <v/>
+      </c>
+      <c r="F49" t="str">
+        <v/>
+      </c>
+      <c r="G49" t="str">
+        <v/>
+      </c>
+      <c r="H49" t="str">
+        <v/>
+      </c>
+      <c r="I49" t="str">
+        <v/>
+      </c>
+      <c r="J49" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O48"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M49"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>